<commit_message>
Preview before sending, live preview card, My submissions, logo request
- Preview step: the project pop-up as visitors will see it, its place on the map
  (state counts before and after, IASC gaps filled), what stays private, then send
- Live preview card on the form, filled in as people type
- My submissions tab: projects sent from this browser, saved only in the browser,
  with a notice about clearing browser data and a Published status once on the map
- 'Send it to the Durable Solutions Unit' wording
- Organisations new to the map are asked to attach their logo (preview, email, template)
- Shared drawing code (render.js) so previews match the published pop-up
</commit_message>
<xml_diff>
--- a/assets/templates/solutions-footprint-projects-template.xlsx
+++ b/assets/templates/solutions-footprint-projects-template.xlsx
@@ -403,7 +403,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="537">
   <si>
     <t xml:space="preserve">Solutions Footprint | Durable Solutions Hub | Sudan</t>
   </si>
@@ -429,10 +429,13 @@
     <t xml:space="preserve">5. Funding towards durable solutions is calculated for you from the budget and the share. The share is self-assessed by your organisation.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Save the file and email it to dswg.sd@undp.org. Attach up to 3 photos per project (JPG or PNG, under 1 MB each), named with the project name. By attaching photos, you confirm you have consent from the people shown to publish them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. The Durable Solutions Unit reviews every project, may contact the focal point, and confirms when projects are published.</t>
+    <t xml:space="preserve">6. Save the file and email it to the Durable Solutions Unit at dswg.sd@undp.org. Attach up to 3 photos per project (JPG or PNG, under 1 MB each), named with the project name. By attaching photos, you confirm you have consent from the people shown to publish them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. First project from your organisation on the map? Please also attach your organisation's logo (PNG or SVG) to the email, so it appears on the map.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. The Durable Solutions Unit reviews every project, may contact the focal point, and confirms when projects are published.</t>
   </si>
   <si>
     <t xml:space="preserve">What is published</t>
@@ -2620,7 +2623,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C70"/>
+  <dimension ref="B1:C71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2687,160 +2690,158 @@
       </c>
       <c r="C17" s="4"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C18" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="3"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="4"/>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="s">
+      <c r="C23" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="C25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="6" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="6" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="3" t="s">
+      <c r="C31" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="5" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>28</v>
-      </c>
+      <c r="C33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="6" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="5" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2848,95 +2849,95 @@
         <v>43</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C43" s="6" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="5" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
-        <v>18</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="6" t="s">
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="6" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="5" t="s">
+      <c r="C49" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="6" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="5" t="s">
+      <c r="C51" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C52" s="6" t="s">
+    </row>
+    <row r="53" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="5" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="5" t="s">
+      <c r="C53" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2944,23 +2945,23 @@
         <v>65</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2968,46 +2969,48 @@
         <v>70</v>
       </c>
       <c r="C57" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="58" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="5" t="s">
+      <c r="C58" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C58" s="6" t="s">
+    </row>
+    <row r="59" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B59" s="5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="5" t="s">
+      <c r="C59" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C59" s="6" t="s">
+    </row>
+    <row r="60" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="5" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C62" s="6"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="5" t="s">
@@ -3043,17 +3046,23 @@
       <c r="B68" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="6"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="5" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="7" t="s">
+      <c r="C69" s="6" t="s">
         <v>88</v>
       </c>
     </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B11:C11"/>
@@ -3064,11 +3073,12 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B33:C33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3116,112 +3126,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="R1" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S1" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X1" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Y1" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Z1" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AA1" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AB1" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AC1" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AD1" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AE1" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AF1" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AG1" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AH1" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AI1" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AJ1" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3841,7 +3851,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3949,953 +3959,953 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="L2" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="I2" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="J2" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="K2" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>103</v>
-      </c>
       <c r="M2" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B3" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="L3" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>124</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>115</v>
-      </c>
       <c r="M3" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D4" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="G4" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="J4" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="L4" s="18" t="s">
-        <v>126</v>
-      </c>
       <c r="M4" s="18" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D5" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="L5" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="F5" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>135</v>
-      </c>
       <c r="M5" s="18" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D6" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="L6" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="F6" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>142</v>
-      </c>
       <c r="M6" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D8" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D10" s="18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F14" s="18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F15" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F16" s="18" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F17" s="18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F18" s="18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F19" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G23" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G24" s="18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G25" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G26" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G27" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G28" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G29" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G30" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G31" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G32" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G33" s="18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H33" s="18" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G34" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G35" s="18" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H35" s="18" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G36" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H36" s="18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G37" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H37" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G38" s="18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H38" s="18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G39" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G40" s="18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H40" s="18" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G41" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G42" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H42" s="18" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G43" s="18" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G44" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H44" s="18" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G45" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G46" s="18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H46" s="18" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G47" s="18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G48" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G49" s="18" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G50" s="18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G51" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G52" s="18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G53" s="18" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G54" s="18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G55" s="18" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G56" s="18" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G57" s="18" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G58" s="18" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G59" s="18" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G60" s="18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G61" s="18" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H61" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G62" s="18" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G63" s="18" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G64" s="18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H64" s="18" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G65" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G66" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G67" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G68" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G69" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G70" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G71" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G72" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H72" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G73" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G74" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H74" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G75" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G76" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G77" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H77" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G78" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H78" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G79" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H79" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H80" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H81" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H82" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H83" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H84" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H85" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H86" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H87" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H88" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H89" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H90" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H91" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H92" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H93" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H94" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H95" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H96" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -4923,664 +4933,664 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="P1" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="Q1" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L2" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="P2" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="R2" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="P3" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="O5" s="18" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P5" s="18" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="Q5" s="18" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="R5" s="18" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="O6" s="18" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="P6" s="18" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="Q6" s="18" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="R6" s="18" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="P7" s="18" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="Q7" s="18" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="R7" s="18" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O8" s="18" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="P8" s="18" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="Q8" s="18" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="R8" s="18" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="O9" s="18" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="P9" s="18" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="Q9" s="18" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="R9" s="18" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="18" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="Q10" s="18" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="R10" s="18" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="18" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="O11" s="18" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="Q11" s="18" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="18" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="O12" s="18" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="O13" s="18" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="Q13" s="18" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H14" s="18" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="O14" s="18" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H15" s="18" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="O15" s="18" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q15" s="18" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H16" s="18" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="O16" s="18" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H17" s="18" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="N17" s="18" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="O17" s="18" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H18" s="18" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="O18" s="18" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N19" s="18" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N20" s="18" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N21" s="18" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N22" s="18" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Template: file details show Microsoft Excel; optional recalculation step
</commit_message>
<xml_diff>
--- a/assets/templates/solutions-footprint-projects-template.xlsx
+++ b/assets/templates/solutions-footprint-projects-template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -24,11 +24,6 @@
     <definedName function="false" hidden="false" name="TypeMap" vbProcedure="false">Lists!$L$2:$M$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
Several donors with amounts on the form, the Excel template and the admin pages
- Form: one row per donor with its amount; with more than one donor every amount is required, and the total cannot exceed the budget
- Excel template: Donor 1 to 3, each with an amount (older copies with one donor column still load)
- Map: donor filter, search and the funding chart handle several donors, splitting funding by their amounts
- Back end and admin pages store and check donors with amounts
</commit_message>
<xml_diff>
--- a/assets/templates/solutions-footprint-projects-template.xlsx
+++ b/assets/templates/solutions-footprint-projects-template.xlsx
@@ -365,7 +365,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Optional.</t>
+          <t xml:space="preserve">Optional. The donor or funding source. If more than one donor funds the project, use Donor 2 and Donor 3 and give the amount from each.</t>
         </r>
       </text>
     </comment>
@@ -377,11 +377,71 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Optional. A second donor.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Needed when there is more than one donor.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Optional. A third donor. More than three: add a second row in a new file, or email the Durable Solutions Unit.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Needed when there is more than one donor.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">Leave empty if not known.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0">
+    <comment ref="AO1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -398,7 +458,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="546">
   <si>
     <t xml:space="preserve">Solutions Footprint | Durable Solutions Hub | Sudan</t>
   </si>
@@ -631,10 +691,37 @@
     <t xml:space="preserve">Calculated automatically. Do not type here.</t>
   </si>
   <si>
-    <t xml:space="preserve">Donor or funding source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional.</t>
+    <t xml:space="preserve">Donor 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. The donor or funding source. If more than one donor funds the project, use Donor 2 and Donor 3 and give the amount from each.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 1 amount (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. A second donor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 2 amount (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needed when there is more than one donor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. A third donor. More than three: add a second row in a new file, or email the Durable Solutions Unit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 3 amount (USD)</t>
   </si>
   <si>
     <t xml:space="preserve">People reached, planned: total</t>
@@ -2618,7 +2705,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C71"/>
+  <dimension ref="B1:C76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2991,7 +3078,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="5" t="s">
         <v>77</v>
       </c>
@@ -3011,49 +3098,89 @@
       <c r="B63" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C63" s="6"/>
+      <c r="C63" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C64" s="6"/>
+        <v>83</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C65" s="6"/>
+        <v>85</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C66" s="6"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C67" s="6"/>
+        <v>88</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C68" s="6"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>88</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C69" s="6"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C70" s="6"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="7" t="s">
-        <v>89</v>
+      <c r="B71" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C71" s="6"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C72" s="6"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C73" s="6"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="7" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -3092,7 +3219,7 @@
     <tabColor rgb="FF1F4E79"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AJ18"/>
+  <dimension ref="A1:AO18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="40"/>
@@ -3110,13 +3237,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="30" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="35" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3211,22 +3342,37 @@
         <v>81</v>
       </c>
       <c r="AE1" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AF1" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AG1" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="AH1" s="8" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="AI1" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="AJ1" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
+      </c>
+      <c r="AK1" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AL1" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="AM1" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AO1" s="8" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3261,14 +3407,19 @@
         <v/>
       </c>
       <c r="AB2" s="10"/>
-      <c r="AC2" s="15"/>
-      <c r="AD2" s="15"/>
-      <c r="AE2" s="15"/>
-      <c r="AF2" s="15"/>
-      <c r="AG2" s="15"/>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="12"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="12"/>
       <c r="AH2" s="15"/>
-      <c r="AI2" s="9"/>
-      <c r="AJ2" s="10"/>
+      <c r="AI2" s="15"/>
+      <c r="AJ2" s="15"/>
+      <c r="AK2" s="15"/>
+      <c r="AL2" s="15"/>
+      <c r="AM2" s="15"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9"/>
@@ -3302,14 +3453,19 @@
         <v/>
       </c>
       <c r="AB3" s="10"/>
-      <c r="AC3" s="15"/>
-      <c r="AD3" s="15"/>
-      <c r="AE3" s="15"/>
-      <c r="AF3" s="15"/>
-      <c r="AG3" s="15"/>
+      <c r="AC3" s="12"/>
+      <c r="AD3" s="10"/>
+      <c r="AE3" s="12"/>
+      <c r="AF3" s="10"/>
+      <c r="AG3" s="12"/>
       <c r="AH3" s="15"/>
-      <c r="AI3" s="9"/>
-      <c r="AJ3" s="10"/>
+      <c r="AI3" s="15"/>
+      <c r="AJ3" s="15"/>
+      <c r="AK3" s="15"/>
+      <c r="AL3" s="15"/>
+      <c r="AM3" s="15"/>
+      <c r="AN3" s="9"/>
+      <c r="AO3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -3343,14 +3499,19 @@
         <v/>
       </c>
       <c r="AB4" s="10"/>
-      <c r="AC4" s="15"/>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
-      <c r="AF4" s="15"/>
-      <c r="AG4" s="15"/>
+      <c r="AC4" s="12"/>
+      <c r="AD4" s="10"/>
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="10"/>
+      <c r="AG4" s="12"/>
       <c r="AH4" s="15"/>
-      <c r="AI4" s="9"/>
-      <c r="AJ4" s="10"/>
+      <c r="AI4" s="15"/>
+      <c r="AJ4" s="15"/>
+      <c r="AK4" s="15"/>
+      <c r="AL4" s="15"/>
+      <c r="AM4" s="15"/>
+      <c r="AN4" s="9"/>
+      <c r="AO4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9"/>
@@ -3384,14 +3545,19 @@
         <v/>
       </c>
       <c r="AB5" s="10"/>
-      <c r="AC5" s="15"/>
-      <c r="AD5" s="15"/>
-      <c r="AE5" s="15"/>
-      <c r="AF5" s="15"/>
-      <c r="AG5" s="15"/>
+      <c r="AC5" s="12"/>
+      <c r="AD5" s="10"/>
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="10"/>
+      <c r="AG5" s="12"/>
       <c r="AH5" s="15"/>
-      <c r="AI5" s="9"/>
-      <c r="AJ5" s="10"/>
+      <c r="AI5" s="15"/>
+      <c r="AJ5" s="15"/>
+      <c r="AK5" s="15"/>
+      <c r="AL5" s="15"/>
+      <c r="AM5" s="15"/>
+      <c r="AN5" s="9"/>
+      <c r="AO5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9"/>
@@ -3425,14 +3591,19 @@
         <v/>
       </c>
       <c r="AB6" s="10"/>
-      <c r="AC6" s="15"/>
-      <c r="AD6" s="15"/>
-      <c r="AE6" s="15"/>
-      <c r="AF6" s="15"/>
-      <c r="AG6" s="15"/>
+      <c r="AC6" s="12"/>
+      <c r="AD6" s="10"/>
+      <c r="AE6" s="12"/>
+      <c r="AF6" s="10"/>
+      <c r="AG6" s="12"/>
       <c r="AH6" s="15"/>
-      <c r="AI6" s="9"/>
-      <c r="AJ6" s="10"/>
+      <c r="AI6" s="15"/>
+      <c r="AJ6" s="15"/>
+      <c r="AK6" s="15"/>
+      <c r="AL6" s="15"/>
+      <c r="AM6" s="15"/>
+      <c r="AN6" s="9"/>
+      <c r="AO6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9"/>
@@ -3466,14 +3637,19 @@
         <v/>
       </c>
       <c r="AB7" s="10"/>
-      <c r="AC7" s="15"/>
-      <c r="AD7" s="15"/>
-      <c r="AE7" s="15"/>
-      <c r="AF7" s="15"/>
-      <c r="AG7" s="15"/>
+      <c r="AC7" s="12"/>
+      <c r="AD7" s="10"/>
+      <c r="AE7" s="12"/>
+      <c r="AF7" s="10"/>
+      <c r="AG7" s="12"/>
       <c r="AH7" s="15"/>
-      <c r="AI7" s="9"/>
-      <c r="AJ7" s="10"/>
+      <c r="AI7" s="15"/>
+      <c r="AJ7" s="15"/>
+      <c r="AK7" s="15"/>
+      <c r="AL7" s="15"/>
+      <c r="AM7" s="15"/>
+      <c r="AN7" s="9"/>
+      <c r="AO7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9"/>
@@ -3507,14 +3683,19 @@
         <v/>
       </c>
       <c r="AB8" s="10"/>
-      <c r="AC8" s="15"/>
-      <c r="AD8" s="15"/>
-      <c r="AE8" s="15"/>
-      <c r="AF8" s="15"/>
-      <c r="AG8" s="15"/>
+      <c r="AC8" s="12"/>
+      <c r="AD8" s="10"/>
+      <c r="AE8" s="12"/>
+      <c r="AF8" s="10"/>
+      <c r="AG8" s="12"/>
       <c r="AH8" s="15"/>
-      <c r="AI8" s="9"/>
-      <c r="AJ8" s="10"/>
+      <c r="AI8" s="15"/>
+      <c r="AJ8" s="15"/>
+      <c r="AK8" s="15"/>
+      <c r="AL8" s="15"/>
+      <c r="AM8" s="15"/>
+      <c r="AN8" s="9"/>
+      <c r="AO8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9"/>
@@ -3548,14 +3729,19 @@
         <v/>
       </c>
       <c r="AB9" s="10"/>
-      <c r="AC9" s="15"/>
-      <c r="AD9" s="15"/>
-      <c r="AE9" s="15"/>
-      <c r="AF9" s="15"/>
-      <c r="AG9" s="15"/>
+      <c r="AC9" s="12"/>
+      <c r="AD9" s="10"/>
+      <c r="AE9" s="12"/>
+      <c r="AF9" s="10"/>
+      <c r="AG9" s="12"/>
       <c r="AH9" s="15"/>
-      <c r="AI9" s="9"/>
-      <c r="AJ9" s="10"/>
+      <c r="AI9" s="15"/>
+      <c r="AJ9" s="15"/>
+      <c r="AK9" s="15"/>
+      <c r="AL9" s="15"/>
+      <c r="AM9" s="15"/>
+      <c r="AN9" s="9"/>
+      <c r="AO9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9"/>
@@ -3589,14 +3775,19 @@
         <v/>
       </c>
       <c r="AB10" s="10"/>
-      <c r="AC10" s="15"/>
-      <c r="AD10" s="15"/>
-      <c r="AE10" s="15"/>
-      <c r="AF10" s="15"/>
-      <c r="AG10" s="15"/>
+      <c r="AC10" s="12"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="12"/>
+      <c r="AF10" s="10"/>
+      <c r="AG10" s="12"/>
       <c r="AH10" s="15"/>
-      <c r="AI10" s="9"/>
-      <c r="AJ10" s="10"/>
+      <c r="AI10" s="15"/>
+      <c r="AJ10" s="15"/>
+      <c r="AK10" s="15"/>
+      <c r="AL10" s="15"/>
+      <c r="AM10" s="15"/>
+      <c r="AN10" s="9"/>
+      <c r="AO10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9"/>
@@ -3630,14 +3821,19 @@
         <v/>
       </c>
       <c r="AB11" s="10"/>
-      <c r="AC11" s="15"/>
-      <c r="AD11" s="15"/>
-      <c r="AE11" s="15"/>
-      <c r="AF11" s="15"/>
-      <c r="AG11" s="15"/>
+      <c r="AC11" s="12"/>
+      <c r="AD11" s="10"/>
+      <c r="AE11" s="12"/>
+      <c r="AF11" s="10"/>
+      <c r="AG11" s="12"/>
       <c r="AH11" s="15"/>
-      <c r="AI11" s="9"/>
-      <c r="AJ11" s="10"/>
+      <c r="AI11" s="15"/>
+      <c r="AJ11" s="15"/>
+      <c r="AK11" s="15"/>
+      <c r="AL11" s="15"/>
+      <c r="AM11" s="15"/>
+      <c r="AN11" s="9"/>
+      <c r="AO11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9"/>
@@ -3671,14 +3867,19 @@
         <v/>
       </c>
       <c r="AB12" s="10"/>
-      <c r="AC12" s="15"/>
-      <c r="AD12" s="15"/>
-      <c r="AE12" s="15"/>
-      <c r="AF12" s="15"/>
-      <c r="AG12" s="15"/>
+      <c r="AC12" s="12"/>
+      <c r="AD12" s="10"/>
+      <c r="AE12" s="12"/>
+      <c r="AF12" s="10"/>
+      <c r="AG12" s="12"/>
       <c r="AH12" s="15"/>
-      <c r="AI12" s="9"/>
-      <c r="AJ12" s="10"/>
+      <c r="AI12" s="15"/>
+      <c r="AJ12" s="15"/>
+      <c r="AK12" s="15"/>
+      <c r="AL12" s="15"/>
+      <c r="AM12" s="15"/>
+      <c r="AN12" s="9"/>
+      <c r="AO12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9"/>
@@ -3712,14 +3913,19 @@
         <v/>
       </c>
       <c r="AB13" s="10"/>
-      <c r="AC13" s="15"/>
-      <c r="AD13" s="15"/>
-      <c r="AE13" s="15"/>
-      <c r="AF13" s="15"/>
-      <c r="AG13" s="15"/>
+      <c r="AC13" s="12"/>
+      <c r="AD13" s="10"/>
+      <c r="AE13" s="12"/>
+      <c r="AF13" s="10"/>
+      <c r="AG13" s="12"/>
       <c r="AH13" s="15"/>
-      <c r="AI13" s="9"/>
-      <c r="AJ13" s="10"/>
+      <c r="AI13" s="15"/>
+      <c r="AJ13" s="15"/>
+      <c r="AK13" s="15"/>
+      <c r="AL13" s="15"/>
+      <c r="AM13" s="15"/>
+      <c r="AN13" s="9"/>
+      <c r="AO13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9"/>
@@ -3753,14 +3959,19 @@
         <v/>
       </c>
       <c r="AB14" s="10"/>
-      <c r="AC14" s="15"/>
-      <c r="AD14" s="15"/>
-      <c r="AE14" s="15"/>
-      <c r="AF14" s="15"/>
-      <c r="AG14" s="15"/>
+      <c r="AC14" s="12"/>
+      <c r="AD14" s="10"/>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="10"/>
+      <c r="AG14" s="12"/>
       <c r="AH14" s="15"/>
-      <c r="AI14" s="9"/>
-      <c r="AJ14" s="10"/>
+      <c r="AI14" s="15"/>
+      <c r="AJ14" s="15"/>
+      <c r="AK14" s="15"/>
+      <c r="AL14" s="15"/>
+      <c r="AM14" s="15"/>
+      <c r="AN14" s="9"/>
+      <c r="AO14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9"/>
@@ -3794,14 +4005,19 @@
         <v/>
       </c>
       <c r="AB15" s="10"/>
-      <c r="AC15" s="15"/>
-      <c r="AD15" s="15"/>
-      <c r="AE15" s="15"/>
-      <c r="AF15" s="15"/>
-      <c r="AG15" s="15"/>
+      <c r="AC15" s="12"/>
+      <c r="AD15" s="10"/>
+      <c r="AE15" s="12"/>
+      <c r="AF15" s="10"/>
+      <c r="AG15" s="12"/>
       <c r="AH15" s="15"/>
-      <c r="AI15" s="9"/>
-      <c r="AJ15" s="10"/>
+      <c r="AI15" s="15"/>
+      <c r="AJ15" s="15"/>
+      <c r="AK15" s="15"/>
+      <c r="AL15" s="15"/>
+      <c r="AM15" s="15"/>
+      <c r="AN15" s="9"/>
+      <c r="AO15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9"/>
@@ -3835,18 +4051,23 @@
         <v/>
       </c>
       <c r="AB16" s="10"/>
-      <c r="AC16" s="15"/>
-      <c r="AD16" s="15"/>
-      <c r="AE16" s="15"/>
-      <c r="AF16" s="15"/>
-      <c r="AG16" s="15"/>
+      <c r="AC16" s="12"/>
+      <c r="AD16" s="10"/>
+      <c r="AE16" s="12"/>
+      <c r="AF16" s="10"/>
+      <c r="AG16" s="12"/>
       <c r="AH16" s="15"/>
-      <c r="AI16" s="9"/>
-      <c r="AJ16" s="10"/>
+      <c r="AI16" s="15"/>
+      <c r="AJ16" s="15"/>
+      <c r="AK16" s="15"/>
+      <c r="AL16" s="15"/>
+      <c r="AM16" s="15"/>
+      <c r="AN16" s="9"/>
+      <c r="AO16" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -3903,7 +4124,7 @@
       <formula1>Lists!$E$2:$E$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="AJ2:AJ16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="AO2:AO16" type="list">
       <formula1>Lists!$E$2:$E$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3954,953 +4175,953 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="K2" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="L2" s="18" t="s">
-        <v>104</v>
-      </c>
       <c r="M2" s="18" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="K3" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="L3" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="L3" s="18" t="s">
-        <v>116</v>
-      </c>
       <c r="M3" s="18" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D8" s="18" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="18" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D10" s="18" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="18" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="18" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F14" s="18" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F15" s="18" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F16" s="18" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F17" s="18" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F18" s="18" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F19" s="18" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="18" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="18" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="18" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G23" s="18" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G24" s="18" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G25" s="18" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G26" s="18" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G27" s="18" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G28" s="18" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G29" s="18" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G30" s="18" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G31" s="18" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G32" s="18" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G33" s="18" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="H33" s="18" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G34" s="18" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G35" s="18" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="H35" s="18" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G36" s="18" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="H36" s="18" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G37" s="18" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="H37" s="18" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G38" s="18" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="H38" s="18" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G39" s="18" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G40" s="18" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="H40" s="18" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G41" s="18" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G42" s="18" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="H42" s="18" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G43" s="18" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G44" s="18" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="H44" s="18" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G45" s="18" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G46" s="18" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="H46" s="18" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G47" s="18" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G48" s="18" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G49" s="18" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G50" s="18" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G51" s="18" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G52" s="18" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G53" s="18" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G54" s="18" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G55" s="18" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G56" s="18" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G57" s="18" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G58" s="18" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G59" s="18" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G60" s="18" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G61" s="18" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="H61" s="18" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G62" s="18" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G63" s="18" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G64" s="18" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="H64" s="18" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G65" s="18" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G66" s="18" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G67" s="18" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G68" s="18" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G69" s="18" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G70" s="18" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G71" s="18" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G72" s="18" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="H72" s="18" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G73" s="18" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G74" s="18" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="H74" s="18" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G75" s="18" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G76" s="18" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G77" s="18" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="H77" s="18" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G78" s="18" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="H78" s="18" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G79" s="18" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="H79" s="18" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H80" s="18" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H81" s="18" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H82" s="18" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H83" s="18" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H84" s="18" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H85" s="18" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H86" s="18" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H87" s="18" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H88" s="18" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H89" s="18" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H90" s="18" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H91" s="18" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H92" s="18" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H93" s="18" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H94" s="18" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H95" s="18" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H96" s="18" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -4928,664 +5149,664 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
       <c r="P1" s="17" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="Q1" s="17" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>351</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="L2" s="18" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="P2" s="18" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="R2" s="18" t="s">
-        <v>369</v>
+        <v>378</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
       <c r="P3" s="18" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>388</v>
+        <v>397</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>389</v>
+        <v>398</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>390</v>
+        <v>399</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>391</v>
+        <v>400</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>394</v>
+        <v>403</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>396</v>
+        <v>405</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>408</v>
+        <v>417</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>409</v>
+        <v>418</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>412</v>
+        <v>421</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>413</v>
+        <v>422</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>414</v>
+        <v>423</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>415</v>
+        <v>424</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>416</v>
+        <v>425</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>417</v>
+        <v>426</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>418</v>
+        <v>427</v>
       </c>
       <c r="O5" s="18" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="P5" s="18" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
       <c r="Q5" s="18" t="s">
-        <v>421</v>
+        <v>430</v>
       </c>
       <c r="R5" s="18" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>424</v>
+        <v>433</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>427</v>
+        <v>436</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>428</v>
+        <v>437</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>429</v>
+        <v>438</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>430</v>
+        <v>439</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>432</v>
+        <v>441</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>433</v>
+        <v>442</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>435</v>
+        <v>444</v>
       </c>
       <c r="O6" s="18" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="P6" s="18" t="s">
-        <v>437</v>
+        <v>446</v>
       </c>
       <c r="Q6" s="18" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="R6" s="18" t="s">
-        <v>439</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>440</v>
+        <v>449</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>441</v>
+        <v>450</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>443</v>
+        <v>452</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>447</v>
+        <v>456</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>452</v>
+        <v>461</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>453</v>
+        <v>462</v>
       </c>
       <c r="P7" s="18" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
       <c r="Q7" s="18" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="R7" s="18" t="s">
-        <v>456</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
       <c r="O8" s="18" t="s">
-        <v>471</v>
+        <v>480</v>
       </c>
       <c r="P8" s="18" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="Q8" s="18" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
       <c r="R8" s="18" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>477</v>
+        <v>486</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>479</v>
+        <v>488</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>480</v>
+        <v>489</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="O9" s="18" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="P9" s="18" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
       <c r="Q9" s="18" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
       <c r="R9" s="18" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="18" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="Q10" s="18" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="R10" s="18" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="18" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="O11" s="18" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="Q11" s="18" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="18" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="O12" s="18" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>512</v>
+        <v>521</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>513</v>
+        <v>522</v>
       </c>
       <c r="O13" s="18" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="Q13" s="18" t="s">
-        <v>515</v>
+        <v>524</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H14" s="18" t="s">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="O14" s="18" t="s">
-        <v>518</v>
+        <v>527</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>519</v>
+        <v>528</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H15" s="18" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="O15" s="18" t="s">
-        <v>522</v>
+        <v>531</v>
       </c>
       <c r="Q15" s="18" t="s">
-        <v>523</v>
+        <v>532</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H16" s="18" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="O16" s="18" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H17" s="18" t="s">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="N17" s="18" t="s">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="O17" s="18" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H18" s="18" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="O18" s="18" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N19" s="18" t="s">
-        <v>533</v>
+        <v>542</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N20" s="18" t="s">
-        <v>534</v>
+        <v>543</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N21" s="18" t="s">
-        <v>535</v>
+        <v>544</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N22" s="18" t="s">
-        <v>536</v>
+        <v>545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IASC criteria: short explanation in a pop-up on each criterion, with the IASC Framework (2010) as source
- Form: an i next to each criterion opens the explanation; the cards keep their size
- About the data: a What it means column and the source
- Excel template: the eight explanations and the source on the Instructions sheet
</commit_message>
<xml_diff>
--- a/assets/templates/solutions-footprint-projects-template.xlsx
+++ b/assets/templates/solutions-footprint-projects-template.xlsx
@@ -458,7 +458,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="565">
   <si>
     <t xml:space="preserve">Solutions Footprint | Durable Solutions Hub | Sudan</t>
   </si>
@@ -539,6 +539,63 @@
   </si>
   <si>
     <t xml:space="preserve">Ongoing, Pipeline or Ended.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The eight IASC criteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Safety and security</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People live in long-term safety and security, without risk of attacks, violence, harassment or landmines, and can move freely.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Adequate standard of living</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People have at least a minimum level of food, water, housing, health care and basic education, without discrimination.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Access to livelihoods and employment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People can find work or other ways to earn a living that let them meet their basic needs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Housing, land and property</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People can get back their homes, land and property, or receive fair compensation, through mechanisms that work.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Access to documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People can obtain or replace personal and other documents, such as identity cards, birth certificates and property deeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Family reunification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Family members separated by displacement can find each other and reunite if they wish.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Participation in public affairs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People can take part in public affairs and community decisions on an equal footing with residents, including voting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Access to effective remedies and justice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People can seek justice and redress for violations linked to their displacement, including through courts and reparation schemes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IASC Framework on Durable Solutions for Internally Displaced Persons (2010): https://interagencystandingcommittee.org/node/2875</t>
   </si>
   <si>
     <t xml:space="preserve">Columns</t>
@@ -2705,7 +2762,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C76"/>
+  <dimension ref="B1:C87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2862,7 +2919,7 @@
       </c>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="5" t="s">
         <v>28</v>
       </c>
@@ -2870,7 +2927,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
         <v>30</v>
       </c>
@@ -2878,7 +2935,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
         <v>32</v>
       </c>
@@ -2886,7 +2943,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="5" t="s">
         <v>34</v>
       </c>
@@ -2902,57 +2959,47 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="5" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="3"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="5" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>48</v>
@@ -2966,7 +3013,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="5" t="s">
         <v>51</v>
       </c>
@@ -2974,7 +3021,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="5" t="s">
         <v>53</v>
       </c>
@@ -2990,201 +3037,289 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="6" t="s">
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="52" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="5" t="s">
+      <c r="C52" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C52" s="6" t="s">
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="5" t="s">
-        <v>63</v>
-      </c>
       <c r="C53" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C55" s="6" t="s">
+    </row>
+    <row r="56" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C57" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="5" t="s">
+      <c r="C58" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C59" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C59" s="6" t="s">
+    </row>
+    <row r="60" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B60" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C60" s="6" t="s">
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="5" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="61" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="5" t="s">
+      <c r="C61" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C62" s="6" t="s">
+    </row>
+    <row r="63" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B63" s="5" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="5" t="s">
+      <c r="C63" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C63" s="6" t="s">
+    </row>
+    <row r="64" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B64" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="5" t="s">
+      <c r="C64" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C67" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C68" s="6"/>
+        <v>89</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C69" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C69" s="6"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="70" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C70" s="6"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C70" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C71" s="6"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>94</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C72" s="6"/>
+        <v>96</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C73" s="6"/>
+        <v>98</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>97</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="7" t="s">
-        <v>98</v>
+      <c r="B76" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C79" s="6"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C81" s="6"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C82" s="6"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C83" s="6"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C84" s="6"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="7" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B11:C11"/>
@@ -3201,6 +3336,7 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B44:C44"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3252,127 +3388,127 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>19</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="R1" s="8" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="S1" s="8" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="T1" s="8" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="U1" s="8" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="W1" s="8" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="X1" s="8" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="Y1" s="8" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="Z1" s="8" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="AA1" s="8" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="AB1" s="8" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="AC1" s="8" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="AD1" s="8" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="AE1" s="8" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="AF1" s="8" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="AG1" s="8" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="AH1" s="8" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AI1" s="8" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AJ1" s="8" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AK1" s="8" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="AL1" s="8" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="AM1" s="8" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="AN1" s="8" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="AO1" s="8" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,7 +4203,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -4175,953 +4311,953 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="L2" s="18" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D8" s="18" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="18" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D10" s="18" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="18" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="18" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F14" s="18" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F15" s="18" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F16" s="18" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F17" s="18" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F18" s="18" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F19" s="18" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="18" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="18" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="18" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G23" s="18" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G24" s="18" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G25" s="18" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G26" s="18" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G27" s="18" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G28" s="18" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G29" s="18" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G30" s="18" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G31" s="18" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G32" s="18" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G33" s="18" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="H33" s="18" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G34" s="18" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G35" s="18" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="H35" s="18" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G36" s="18" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="H36" s="18" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G37" s="18" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="H37" s="18" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G38" s="18" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="H38" s="18" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G39" s="18" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G40" s="18" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="H40" s="18" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G41" s="18" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G42" s="18" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="H42" s="18" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G43" s="18" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G44" s="18" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="H44" s="18" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G45" s="18" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G46" s="18" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="H46" s="18" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G47" s="18" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G48" s="18" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G49" s="18" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G50" s="18" t="s">
-        <v>266</v>
+        <v>285</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G51" s="18" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G52" s="18" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G53" s="18" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G54" s="18" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G55" s="18" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G56" s="18" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G57" s="18" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G58" s="18" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G59" s="18" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G60" s="18" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G61" s="18" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="H61" s="18" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G62" s="18" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G63" s="18" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G64" s="18" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="H64" s="18" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G65" s="18" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G66" s="18" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G67" s="18" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G68" s="18" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G69" s="18" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G70" s="18" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>307</v>
+        <v>326</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G71" s="18" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G72" s="18" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="H72" s="18" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G73" s="18" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G74" s="18" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="H74" s="18" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G75" s="18" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G76" s="18" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G77" s="18" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="H77" s="18" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G78" s="18" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="H78" s="18" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G79" s="18" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="H79" s="18" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H80" s="18" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H81" s="18" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H82" s="18" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H83" s="18" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H84" s="18" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H85" s="18" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H86" s="18" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H87" s="18" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H88" s="18" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H89" s="18" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H90" s="18" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H91" s="18" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H92" s="18" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H93" s="18" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H94" s="18" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H95" s="18" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H96" s="18" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -5149,664 +5285,664 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="P1" s="17" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="Q1" s="17" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>371</v>
+        <v>390</v>
       </c>
       <c r="L2" s="18" t="s">
-        <v>372</v>
+        <v>391</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>373</v>
+        <v>392</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>374</v>
+        <v>393</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="P2" s="18" t="s">
-        <v>376</v>
+        <v>395</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="R2" s="18" t="s">
-        <v>378</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>379</v>
+        <v>398</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>380</v>
+        <v>399</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>381</v>
+        <v>400</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>383</v>
+        <v>402</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>384</v>
+        <v>403</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>385</v>
+        <v>404</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>386</v>
+        <v>405</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>387</v>
+        <v>406</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>389</v>
+        <v>408</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>390</v>
+        <v>409</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>391</v>
+        <v>410</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>392</v>
+        <v>411</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>393</v>
+        <v>412</v>
       </c>
       <c r="P3" s="18" t="s">
-        <v>394</v>
+        <v>413</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>395</v>
+        <v>414</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>396</v>
+        <v>415</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>397</v>
+        <v>416</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>398</v>
+        <v>417</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>399</v>
+        <v>418</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>400</v>
+        <v>419</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>402</v>
+        <v>421</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>403</v>
+        <v>422</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>405</v>
+        <v>424</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>407</v>
+        <v>426</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>408</v>
+        <v>427</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>409</v>
+        <v>428</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>410</v>
+        <v>429</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>412</v>
+        <v>431</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>413</v>
+        <v>432</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>414</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>415</v>
+        <v>434</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>417</v>
+        <v>436</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>418</v>
+        <v>437</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>419</v>
+        <v>438</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>420</v>
+        <v>439</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>421</v>
+        <v>440</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>422</v>
+        <v>441</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>423</v>
+        <v>442</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>424</v>
+        <v>443</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>425</v>
+        <v>444</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>426</v>
+        <v>445</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>427</v>
+        <v>446</v>
       </c>
       <c r="O5" s="18" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="P5" s="18" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="Q5" s="18" t="s">
-        <v>430</v>
+        <v>449</v>
       </c>
       <c r="R5" s="18" t="s">
-        <v>431</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>432</v>
+        <v>451</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>433</v>
+        <v>452</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>434</v>
+        <v>453</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>435</v>
+        <v>454</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>436</v>
+        <v>455</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>437</v>
+        <v>456</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>438</v>
+        <v>457</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>439</v>
+        <v>458</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>440</v>
+        <v>459</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>441</v>
+        <v>460</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>443</v>
+        <v>462</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>444</v>
+        <v>463</v>
       </c>
       <c r="O6" s="18" t="s">
-        <v>445</v>
+        <v>464</v>
       </c>
       <c r="P6" s="18" t="s">
-        <v>446</v>
+        <v>465</v>
       </c>
       <c r="Q6" s="18" t="s">
-        <v>447</v>
+        <v>466</v>
       </c>
       <c r="R6" s="18" t="s">
-        <v>448</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>452</v>
+        <v>471</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>453</v>
+        <v>472</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>454</v>
+        <v>473</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>455</v>
+        <v>474</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>456</v>
+        <v>475</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>457</v>
+        <v>476</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>458</v>
+        <v>477</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>459</v>
+        <v>478</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>460</v>
+        <v>479</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>461</v>
+        <v>480</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>462</v>
+        <v>481</v>
       </c>
       <c r="P7" s="18" t="s">
-        <v>463</v>
+        <v>482</v>
       </c>
       <c r="Q7" s="18" t="s">
-        <v>464</v>
+        <v>483</v>
       </c>
       <c r="R7" s="18" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>466</v>
+        <v>485</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>467</v>
+        <v>486</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>468</v>
+        <v>487</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>469</v>
+        <v>488</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>470</v>
+        <v>489</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>472</v>
+        <v>491</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>473</v>
+        <v>492</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>476</v>
+        <v>495</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>478</v>
+        <v>497</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="O8" s="18" t="s">
-        <v>480</v>
+        <v>499</v>
       </c>
       <c r="P8" s="18" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="Q8" s="18" t="s">
-        <v>482</v>
+        <v>501</v>
       </c>
       <c r="R8" s="18" t="s">
-        <v>483</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>484</v>
+        <v>503</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>485</v>
+        <v>504</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>487</v>
+        <v>506</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>489</v>
+        <v>508</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>490</v>
+        <v>509</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>491</v>
+        <v>510</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>492</v>
+        <v>511</v>
       </c>
       <c r="O9" s="18" t="s">
-        <v>493</v>
+        <v>512</v>
       </c>
       <c r="P9" s="18" t="s">
-        <v>494</v>
+        <v>513</v>
       </c>
       <c r="Q9" s="18" t="s">
-        <v>495</v>
+        <v>514</v>
       </c>
       <c r="R9" s="18" t="s">
-        <v>496</v>
+        <v>515</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="18" t="s">
-        <v>497</v>
+        <v>516</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>499</v>
+        <v>518</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>501</v>
+        <v>520</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>503</v>
+        <v>522</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>504</v>
+        <v>523</v>
       </c>
       <c r="Q10" s="18" t="s">
-        <v>505</v>
+        <v>524</v>
       </c>
       <c r="R10" s="18" t="s">
-        <v>506</v>
+        <v>525</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="18" t="s">
-        <v>507</v>
+        <v>526</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>508</v>
+        <v>527</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>509</v>
+        <v>528</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>510</v>
+        <v>529</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="O11" s="18" t="s">
-        <v>512</v>
+        <v>531</v>
       </c>
       <c r="Q11" s="18" t="s">
-        <v>513</v>
+        <v>532</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="18" t="s">
-        <v>514</v>
+        <v>533</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>515</v>
+        <v>534</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>516</v>
+        <v>535</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>517</v>
+        <v>536</v>
       </c>
       <c r="O12" s="18" t="s">
-        <v>518</v>
+        <v>537</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>519</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F13" s="18" t="s">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>521</v>
+        <v>540</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="O13" s="18" t="s">
-        <v>523</v>
+        <v>542</v>
       </c>
       <c r="Q13" s="18" t="s">
-        <v>524</v>
+        <v>543</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H14" s="18" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>526</v>
+        <v>545</v>
       </c>
       <c r="O14" s="18" t="s">
-        <v>527</v>
+        <v>546</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H15" s="18" t="s">
-        <v>529</v>
+        <v>548</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="O15" s="18" t="s">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="Q15" s="18" t="s">
-        <v>532</v>
+        <v>551</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H16" s="18" t="s">
-        <v>533</v>
+        <v>552</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>534</v>
+        <v>553</v>
       </c>
       <c r="O16" s="18" t="s">
-        <v>535</v>
+        <v>554</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H17" s="18" t="s">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="N17" s="18" t="s">
-        <v>537</v>
+        <v>556</v>
       </c>
       <c r="O17" s="18" t="s">
-        <v>538</v>
+        <v>557</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H18" s="18" t="s">
-        <v>539</v>
+        <v>558</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>540</v>
+        <v>559</v>
       </c>
       <c r="O18" s="18" t="s">
-        <v>541</v>
+        <v>560</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N19" s="18" t="s">
-        <v>542</v>
+        <v>561</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N20" s="18" t="s">
-        <v>543</v>
+        <v>562</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N21" s="18" t="s">
-        <v>544</v>
+        <v>563</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N22" s="18" t="s">
-        <v>545</v>
+        <v>564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
People reached: total adds up the groups, women and girls share, persons with disabilities, optional breakdown; up to 5 donors
- Form: total calculated from the groups; people reached and the share of women and girls required; persons with disabilities share with the share of women and girls among them; optional breakdown by women, girls, men and boys per group; whole-number checks
- Excel template: five donor pairs, the new people columns, total calculated, the 20 breakdown columns folded away
- Upload page, data script, back end and admin pages read and store the new fields
</commit_message>
<xml_diff>
--- a/assets/templates/solutions-footprint-projects-template.xlsx
+++ b/assets/templates/solutions-footprint-projects-template.xlsx
@@ -365,7 +365,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Optional. The donor or funding source. If more than one donor funds the project, use Donor 2 and Donor 3 and give the amount from each.</t>
+          <t xml:space="preserve">Optional. The donor or funding source.</t>
         </r>
       </text>
     </comment>
@@ -389,7 +389,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Optional. A second donor.</t>
+          <t xml:space="preserve">Optional. Donor 2 (up to 5 donors per project).</t>
         </r>
       </text>
     </comment>
@@ -401,7 +401,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Needed when there is more than one donor.</t>
+          <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
         </r>
       </text>
     </comment>
@@ -413,7 +413,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Optional. A third donor. More than three: add a second row in a new file, or email the Durable Solutions Unit.</t>
+          <t xml:space="preserve">Optional. Donor 3 (up to 5 donors per project).</t>
         </r>
       </text>
     </comment>
@@ -425,7 +425,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Needed when there is more than one donor.</t>
+          <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
         </r>
       </text>
     </comment>
@@ -437,11 +437,155 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Leave empty if not known.</t>
+          <t xml:space="preserve">Optional. Donor 4 (up to 5 donors per project).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Optional. Donor 5 (up to 5 donors per project).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Needed when there is more than one donor. Number in US dollars, without the $ sign.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AL1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Number of IDPs reached, planned. At least one group is required.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AM1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Number of returnees.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AN1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Number of refugees.</t>
         </r>
       </text>
     </comment>
     <comment ref="AO1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Number of people in the host community.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AP1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">People not in a group above. If you only know the total, enter it here.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AQ1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Adds up the five groups. Do not type here.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AR1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Share of all people reached, from 0 to 100. If you fill in the breakdown by women, girls, men and boys, it is calculated from that instead.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AS1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Optional. Share of all people reached, from 0 to 100.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AT1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Optional. Share of women and girls among persons with disabilities, from 0 to 100.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BP1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -458,7 +602,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="604">
   <si>
     <t xml:space="preserve">Solutions Footprint | Durable Solutions Hub | Sudan</t>
   </si>
@@ -751,7 +895,7 @@
     <t xml:space="preserve">Donor 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional. The donor or funding source. If more than one donor funds the project, use Donor 2 and Donor 3 and give the amount from each.</t>
+    <t xml:space="preserve">Optional. The donor or funding source.</t>
   </si>
   <si>
     <t xml:space="preserve">Donor 1 amount (USD)</t>
@@ -763,232 +907,349 @@
     <t xml:space="preserve">Donor 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional. A second donor.</t>
+    <t xml:space="preserve">Optional. Donor 2 (up to 5 donors per project).</t>
   </si>
   <si>
     <t xml:space="preserve">Donor 2 amount (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Needed when there is more than one donor.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Donor 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional. A third donor. More than three: add a second row in a new file, or email the Durable Solutions Unit.</t>
+    <t xml:space="preserve">Optional. Donor 3 (up to 5 donors per project).</t>
   </si>
   <si>
     <t xml:space="preserve">Donor 3 amount (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">People reached, planned: total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leave empty if not known.</t>
+    <t xml:space="preserve">Donor 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Donor 4 (up to 5 donors per project).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 4 amount (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Donor 5 (up to 5 donors per project).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donor 5 amount (USD)</t>
   </si>
   <si>
     <t xml:space="preserve">IDPs</t>
   </si>
   <si>
+    <t xml:space="preserve">Number of IDPs reached, planned. At least one group is required.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Returnees</t>
   </si>
   <si>
+    <t xml:space="preserve">Number of returnees.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Refugees</t>
   </si>
   <si>
+    <t xml:space="preserve">Number of refugees.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Host community</t>
   </si>
   <si>
+    <t xml:space="preserve">Number of people in the host community.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other or not specified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People not in a group above. If you only know the total, enter it here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total people (calculated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adds up the five groups. Do not type here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Women and girls (%) *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of all people reached, from 0 to 100. If you fill in the breakdown by women, girls, men and boys, it is calculated from that instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persons with disabilities (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Share of all people reached, from 0 to 100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Of whom women and girls (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Share of women and girls among persons with disabilities, from 0 to 100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remarks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consent to publish *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write Yes to confirm the information can be published on the United Nations in Sudan website.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breakdown by women, girls, men and boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. These 20 columns are folded away after 'Of whom women and girls (%)': click the + above the column letters to open them. For each group, give the number of women, girls, men and boys (girls and boys are under 18). When a group has a breakdown, its number should equal the sum of the breakdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questions: dswg.sd@undp.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDPs: women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDPs: girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDPs: men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDPs: boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returnees: women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returnees: girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returnees: men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returnees: boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refugees: women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refugees: girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refugees: men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refugees: boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host community: women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host community: girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host community: men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host community: boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other or not specified: women</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other or not specified: girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other or not specified: men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other or not specified: boys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need more rows? Copy the last row and paste it below, or send a second file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organisation types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geographic scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordination mechanism</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UN agency (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International NGO (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National NGO (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red Cross / Red Crescent (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authorities (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other (acronym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UN agency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongoing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nationwide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durable Solutions Working Group (DSWG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRUZROJA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MoE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orgs_UN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choose the organisation type first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International NGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pipeline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One or more states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area Durable Solutions Working Group (ADSWG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAR JAPAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MoH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orgs_INGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National NGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information Management Working Group (IMWG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ILO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGWA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SpRC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOPER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orgs_NNGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red Cross / Red Crescent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protection Cluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACF-Spain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AHSWCD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orgs_RC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authorities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shelter Cluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCHA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act Appeal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orgs_Auth</t>
+  </si>
+  <si>
     <t xml:space="preserve">Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remarks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consent to publish *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write Yes to confirm the information can be published on the United Nations in Sudan website.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Questions: dswg.sd@undp.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Need more rows? Copy the last row and paste it below, or send a second file.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organisation types</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geographic scope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coordination mechanism</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UN agency (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">International NGO (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National NGO (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Red Cross / Red Crescent (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authorities (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other (acronym)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">List name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UN agency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ongoing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nationwide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Durable Solutions Working Group (DSWG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRUZROJA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MoE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orgs_UN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Choose the organisation type first</t>
-  </si>
-  <si>
-    <t xml:space="preserve">International NGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pipeline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One or more states</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Area Durable Solutions Working Group (ADSWG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AAR JAPAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MoH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orgs_INGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National NGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Management Working Group (IMWG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ILO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGWA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SpRC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOPER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orgs_NNGO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Red Cross / Red Crescent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protection Cluster</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACF-Spain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AHSWCD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orgs_RC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authorities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shelter Cluster</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCHA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Act Appeal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orgs_Auth</t>
   </si>
   <si>
     <t xml:space="preserve">Health Cluster</t>
@@ -2159,12 +2420,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="\$#,##0"/>
     <numFmt numFmtId="167" formatCode="0%"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="0"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -2353,7 +2615,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2415,6 +2677,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2762,7 +3032,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C87"/>
+  <dimension ref="B1:C95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -3213,7 +3483,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="5" t="s">
         <v>96</v>
       </c>
@@ -3242,80 +3512,154 @@
         <v>102</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C76" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C78" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C79" s="6"/>
+        <v>108</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C80" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C80" s="6"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C81" s="6"/>
+      <c r="C81" s="6" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C82" s="6"/>
+      <c r="C82" s="6" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C83" s="6"/>
+        <v>114</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C84" s="6"/>
+        <v>116</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="7" t="s">
-        <v>117</v>
+      <c r="B87" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B88" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B89" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B90" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B91" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C91" s="6"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B92" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B93" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B95" s="7" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3355,8 +3699,8 @@
     <tabColor rgb="FF1F4E79"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AO18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BP18"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
@@ -3378,12 +3722,21 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="35" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="42" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="45" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="66" min="47" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3481,19 +3834,19 @@
         <v>102</v>
       </c>
       <c r="AF1" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AG1" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="AH1" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="AH1" s="8" t="s">
-        <v>107</v>
-      </c>
       <c r="AI1" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="AJ1" s="8" t="s">
         <v>109</v>
-      </c>
-      <c r="AJ1" s="8" t="s">
-        <v>110</v>
       </c>
       <c r="AK1" s="8" t="s">
         <v>111</v>
@@ -3502,13 +3855,94 @@
         <v>112</v>
       </c>
       <c r="AM1" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AN1" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="AO1" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
+      </c>
+      <c r="AP1" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="AQ1" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR1" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="AS1" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="AT1" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="AU1" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="AV1" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="AW1" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="AX1" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="AY1" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="AZ1" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="BA1" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB1" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC1" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="BD1" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="BE1" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="BF1" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="BG1" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="BH1" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="BI1" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="BJ1" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="BK1" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="BL1" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="BM1" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="BN1" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="BO1" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="BP1" s="8" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3548,14 +3982,44 @@
       <c r="AE2" s="12"/>
       <c r="AF2" s="10"/>
       <c r="AG2" s="12"/>
-      <c r="AH2" s="15"/>
-      <c r="AI2" s="15"/>
-      <c r="AJ2" s="15"/>
-      <c r="AK2" s="15"/>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="12"/>
+      <c r="AJ2" s="10"/>
+      <c r="AK2" s="12"/>
       <c r="AL2" s="15"/>
       <c r="AM2" s="15"/>
-      <c r="AN2" s="9"/>
-      <c r="AO2" s="10"/>
+      <c r="AN2" s="15"/>
+      <c r="AO2" s="15"/>
+      <c r="AP2" s="15"/>
+      <c r="AQ2" s="16" t="str">
+        <f aca="false">IF(COUNT(AL2:AP2)=0,"",SUM(AL2:AP2))</f>
+        <v/>
+      </c>
+      <c r="AR2" s="17"/>
+      <c r="AS2" s="17"/>
+      <c r="AT2" s="17"/>
+      <c r="AU2" s="15"/>
+      <c r="AV2" s="15"/>
+      <c r="AW2" s="15"/>
+      <c r="AX2" s="15"/>
+      <c r="AY2" s="15"/>
+      <c r="AZ2" s="15"/>
+      <c r="BA2" s="15"/>
+      <c r="BB2" s="15"/>
+      <c r="BC2" s="15"/>
+      <c r="BD2" s="15"/>
+      <c r="BE2" s="15"/>
+      <c r="BF2" s="15"/>
+      <c r="BG2" s="15"/>
+      <c r="BH2" s="15"/>
+      <c r="BI2" s="15"/>
+      <c r="BJ2" s="15"/>
+      <c r="BK2" s="15"/>
+      <c r="BL2" s="15"/>
+      <c r="BM2" s="15"/>
+      <c r="BN2" s="15"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9"/>
@@ -3594,14 +4058,44 @@
       <c r="AE3" s="12"/>
       <c r="AF3" s="10"/>
       <c r="AG3" s="12"/>
-      <c r="AH3" s="15"/>
-      <c r="AI3" s="15"/>
-      <c r="AJ3" s="15"/>
-      <c r="AK3" s="15"/>
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="12"/>
+      <c r="AJ3" s="10"/>
+      <c r="AK3" s="12"/>
       <c r="AL3" s="15"/>
       <c r="AM3" s="15"/>
-      <c r="AN3" s="9"/>
-      <c r="AO3" s="10"/>
+      <c r="AN3" s="15"/>
+      <c r="AO3" s="15"/>
+      <c r="AP3" s="15"/>
+      <c r="AQ3" s="16" t="str">
+        <f aca="false">IF(COUNT(AL3:AP3)=0,"",SUM(AL3:AP3))</f>
+        <v/>
+      </c>
+      <c r="AR3" s="17"/>
+      <c r="AS3" s="17"/>
+      <c r="AT3" s="17"/>
+      <c r="AU3" s="15"/>
+      <c r="AV3" s="15"/>
+      <c r="AW3" s="15"/>
+      <c r="AX3" s="15"/>
+      <c r="AY3" s="15"/>
+      <c r="AZ3" s="15"/>
+      <c r="BA3" s="15"/>
+      <c r="BB3" s="15"/>
+      <c r="BC3" s="15"/>
+      <c r="BD3" s="15"/>
+      <c r="BE3" s="15"/>
+      <c r="BF3" s="15"/>
+      <c r="BG3" s="15"/>
+      <c r="BH3" s="15"/>
+      <c r="BI3" s="15"/>
+      <c r="BJ3" s="15"/>
+      <c r="BK3" s="15"/>
+      <c r="BL3" s="15"/>
+      <c r="BM3" s="15"/>
+      <c r="BN3" s="15"/>
+      <c r="BO3" s="9"/>
+      <c r="BP3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -3640,14 +4134,44 @@
       <c r="AE4" s="12"/>
       <c r="AF4" s="10"/>
       <c r="AG4" s="12"/>
-      <c r="AH4" s="15"/>
-      <c r="AI4" s="15"/>
-      <c r="AJ4" s="15"/>
-      <c r="AK4" s="15"/>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="10"/>
+      <c r="AK4" s="12"/>
       <c r="AL4" s="15"/>
       <c r="AM4" s="15"/>
-      <c r="AN4" s="9"/>
-      <c r="AO4" s="10"/>
+      <c r="AN4" s="15"/>
+      <c r="AO4" s="15"/>
+      <c r="AP4" s="15"/>
+      <c r="AQ4" s="16" t="str">
+        <f aca="false">IF(COUNT(AL4:AP4)=0,"",SUM(AL4:AP4))</f>
+        <v/>
+      </c>
+      <c r="AR4" s="17"/>
+      <c r="AS4" s="17"/>
+      <c r="AT4" s="17"/>
+      <c r="AU4" s="15"/>
+      <c r="AV4" s="15"/>
+      <c r="AW4" s="15"/>
+      <c r="AX4" s="15"/>
+      <c r="AY4" s="15"/>
+      <c r="AZ4" s="15"/>
+      <c r="BA4" s="15"/>
+      <c r="BB4" s="15"/>
+      <c r="BC4" s="15"/>
+      <c r="BD4" s="15"/>
+      <c r="BE4" s="15"/>
+      <c r="BF4" s="15"/>
+      <c r="BG4" s="15"/>
+      <c r="BH4" s="15"/>
+      <c r="BI4" s="15"/>
+      <c r="BJ4" s="15"/>
+      <c r="BK4" s="15"/>
+      <c r="BL4" s="15"/>
+      <c r="BM4" s="15"/>
+      <c r="BN4" s="15"/>
+      <c r="BO4" s="9"/>
+      <c r="BP4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9"/>
@@ -3686,14 +4210,44 @@
       <c r="AE5" s="12"/>
       <c r="AF5" s="10"/>
       <c r="AG5" s="12"/>
-      <c r="AH5" s="15"/>
-      <c r="AI5" s="15"/>
-      <c r="AJ5" s="15"/>
-      <c r="AK5" s="15"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="12"/>
+      <c r="AJ5" s="10"/>
+      <c r="AK5" s="12"/>
       <c r="AL5" s="15"/>
       <c r="AM5" s="15"/>
-      <c r="AN5" s="9"/>
-      <c r="AO5" s="10"/>
+      <c r="AN5" s="15"/>
+      <c r="AO5" s="15"/>
+      <c r="AP5" s="15"/>
+      <c r="AQ5" s="16" t="str">
+        <f aca="false">IF(COUNT(AL5:AP5)=0,"",SUM(AL5:AP5))</f>
+        <v/>
+      </c>
+      <c r="AR5" s="17"/>
+      <c r="AS5" s="17"/>
+      <c r="AT5" s="17"/>
+      <c r="AU5" s="15"/>
+      <c r="AV5" s="15"/>
+      <c r="AW5" s="15"/>
+      <c r="AX5" s="15"/>
+      <c r="AY5" s="15"/>
+      <c r="AZ5" s="15"/>
+      <c r="BA5" s="15"/>
+      <c r="BB5" s="15"/>
+      <c r="BC5" s="15"/>
+      <c r="BD5" s="15"/>
+      <c r="BE5" s="15"/>
+      <c r="BF5" s="15"/>
+      <c r="BG5" s="15"/>
+      <c r="BH5" s="15"/>
+      <c r="BI5" s="15"/>
+      <c r="BJ5" s="15"/>
+      <c r="BK5" s="15"/>
+      <c r="BL5" s="15"/>
+      <c r="BM5" s="15"/>
+      <c r="BN5" s="15"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9"/>
@@ -3732,14 +4286,44 @@
       <c r="AE6" s="12"/>
       <c r="AF6" s="10"/>
       <c r="AG6" s="12"/>
-      <c r="AH6" s="15"/>
-      <c r="AI6" s="15"/>
-      <c r="AJ6" s="15"/>
-      <c r="AK6" s="15"/>
+      <c r="AH6" s="10"/>
+      <c r="AI6" s="12"/>
+      <c r="AJ6" s="10"/>
+      <c r="AK6" s="12"/>
       <c r="AL6" s="15"/>
       <c r="AM6" s="15"/>
-      <c r="AN6" s="9"/>
-      <c r="AO6" s="10"/>
+      <c r="AN6" s="15"/>
+      <c r="AO6" s="15"/>
+      <c r="AP6" s="15"/>
+      <c r="AQ6" s="16" t="str">
+        <f aca="false">IF(COUNT(AL6:AP6)=0,"",SUM(AL6:AP6))</f>
+        <v/>
+      </c>
+      <c r="AR6" s="17"/>
+      <c r="AS6" s="17"/>
+      <c r="AT6" s="17"/>
+      <c r="AU6" s="15"/>
+      <c r="AV6" s="15"/>
+      <c r="AW6" s="15"/>
+      <c r="AX6" s="15"/>
+      <c r="AY6" s="15"/>
+      <c r="AZ6" s="15"/>
+      <c r="BA6" s="15"/>
+      <c r="BB6" s="15"/>
+      <c r="BC6" s="15"/>
+      <c r="BD6" s="15"/>
+      <c r="BE6" s="15"/>
+      <c r="BF6" s="15"/>
+      <c r="BG6" s="15"/>
+      <c r="BH6" s="15"/>
+      <c r="BI6" s="15"/>
+      <c r="BJ6" s="15"/>
+      <c r="BK6" s="15"/>
+      <c r="BL6" s="15"/>
+      <c r="BM6" s="15"/>
+      <c r="BN6" s="15"/>
+      <c r="BO6" s="9"/>
+      <c r="BP6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9"/>
@@ -3778,14 +4362,44 @@
       <c r="AE7" s="12"/>
       <c r="AF7" s="10"/>
       <c r="AG7" s="12"/>
-      <c r="AH7" s="15"/>
-      <c r="AI7" s="15"/>
-      <c r="AJ7" s="15"/>
-      <c r="AK7" s="15"/>
+      <c r="AH7" s="10"/>
+      <c r="AI7" s="12"/>
+      <c r="AJ7" s="10"/>
+      <c r="AK7" s="12"/>
       <c r="AL7" s="15"/>
       <c r="AM7" s="15"/>
-      <c r="AN7" s="9"/>
-      <c r="AO7" s="10"/>
+      <c r="AN7" s="15"/>
+      <c r="AO7" s="15"/>
+      <c r="AP7" s="15"/>
+      <c r="AQ7" s="16" t="str">
+        <f aca="false">IF(COUNT(AL7:AP7)=0,"",SUM(AL7:AP7))</f>
+        <v/>
+      </c>
+      <c r="AR7" s="17"/>
+      <c r="AS7" s="17"/>
+      <c r="AT7" s="17"/>
+      <c r="AU7" s="15"/>
+      <c r="AV7" s="15"/>
+      <c r="AW7" s="15"/>
+      <c r="AX7" s="15"/>
+      <c r="AY7" s="15"/>
+      <c r="AZ7" s="15"/>
+      <c r="BA7" s="15"/>
+      <c r="BB7" s="15"/>
+      <c r="BC7" s="15"/>
+      <c r="BD7" s="15"/>
+      <c r="BE7" s="15"/>
+      <c r="BF7" s="15"/>
+      <c r="BG7" s="15"/>
+      <c r="BH7" s="15"/>
+      <c r="BI7" s="15"/>
+      <c r="BJ7" s="15"/>
+      <c r="BK7" s="15"/>
+      <c r="BL7" s="15"/>
+      <c r="BM7" s="15"/>
+      <c r="BN7" s="15"/>
+      <c r="BO7" s="9"/>
+      <c r="BP7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9"/>
@@ -3824,14 +4438,44 @@
       <c r="AE8" s="12"/>
       <c r="AF8" s="10"/>
       <c r="AG8" s="12"/>
-      <c r="AH8" s="15"/>
-      <c r="AI8" s="15"/>
-      <c r="AJ8" s="15"/>
-      <c r="AK8" s="15"/>
+      <c r="AH8" s="10"/>
+      <c r="AI8" s="12"/>
+      <c r="AJ8" s="10"/>
+      <c r="AK8" s="12"/>
       <c r="AL8" s="15"/>
       <c r="AM8" s="15"/>
-      <c r="AN8" s="9"/>
-      <c r="AO8" s="10"/>
+      <c r="AN8" s="15"/>
+      <c r="AO8" s="15"/>
+      <c r="AP8" s="15"/>
+      <c r="AQ8" s="16" t="str">
+        <f aca="false">IF(COUNT(AL8:AP8)=0,"",SUM(AL8:AP8))</f>
+        <v/>
+      </c>
+      <c r="AR8" s="17"/>
+      <c r="AS8" s="17"/>
+      <c r="AT8" s="17"/>
+      <c r="AU8" s="15"/>
+      <c r="AV8" s="15"/>
+      <c r="AW8" s="15"/>
+      <c r="AX8" s="15"/>
+      <c r="AY8" s="15"/>
+      <c r="AZ8" s="15"/>
+      <c r="BA8" s="15"/>
+      <c r="BB8" s="15"/>
+      <c r="BC8" s="15"/>
+      <c r="BD8" s="15"/>
+      <c r="BE8" s="15"/>
+      <c r="BF8" s="15"/>
+      <c r="BG8" s="15"/>
+      <c r="BH8" s="15"/>
+      <c r="BI8" s="15"/>
+      <c r="BJ8" s="15"/>
+      <c r="BK8" s="15"/>
+      <c r="BL8" s="15"/>
+      <c r="BM8" s="15"/>
+      <c r="BN8" s="15"/>
+      <c r="BO8" s="9"/>
+      <c r="BP8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9"/>
@@ -3870,14 +4514,44 @@
       <c r="AE9" s="12"/>
       <c r="AF9" s="10"/>
       <c r="AG9" s="12"/>
-      <c r="AH9" s="15"/>
-      <c r="AI9" s="15"/>
-      <c r="AJ9" s="15"/>
-      <c r="AK9" s="15"/>
+      <c r="AH9" s="10"/>
+      <c r="AI9" s="12"/>
+      <c r="AJ9" s="10"/>
+      <c r="AK9" s="12"/>
       <c r="AL9" s="15"/>
       <c r="AM9" s="15"/>
-      <c r="AN9" s="9"/>
-      <c r="AO9" s="10"/>
+      <c r="AN9" s="15"/>
+      <c r="AO9" s="15"/>
+      <c r="AP9" s="15"/>
+      <c r="AQ9" s="16" t="str">
+        <f aca="false">IF(COUNT(AL9:AP9)=0,"",SUM(AL9:AP9))</f>
+        <v/>
+      </c>
+      <c r="AR9" s="17"/>
+      <c r="AS9" s="17"/>
+      <c r="AT9" s="17"/>
+      <c r="AU9" s="15"/>
+      <c r="AV9" s="15"/>
+      <c r="AW9" s="15"/>
+      <c r="AX9" s="15"/>
+      <c r="AY9" s="15"/>
+      <c r="AZ9" s="15"/>
+      <c r="BA9" s="15"/>
+      <c r="BB9" s="15"/>
+      <c r="BC9" s="15"/>
+      <c r="BD9" s="15"/>
+      <c r="BE9" s="15"/>
+      <c r="BF9" s="15"/>
+      <c r="BG9" s="15"/>
+      <c r="BH9" s="15"/>
+      <c r="BI9" s="15"/>
+      <c r="BJ9" s="15"/>
+      <c r="BK9" s="15"/>
+      <c r="BL9" s="15"/>
+      <c r="BM9" s="15"/>
+      <c r="BN9" s="15"/>
+      <c r="BO9" s="9"/>
+      <c r="BP9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9"/>
@@ -3916,14 +4590,44 @@
       <c r="AE10" s="12"/>
       <c r="AF10" s="10"/>
       <c r="AG10" s="12"/>
-      <c r="AH10" s="15"/>
-      <c r="AI10" s="15"/>
-      <c r="AJ10" s="15"/>
-      <c r="AK10" s="15"/>
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="12"/>
+      <c r="AJ10" s="10"/>
+      <c r="AK10" s="12"/>
       <c r="AL10" s="15"/>
       <c r="AM10" s="15"/>
-      <c r="AN10" s="9"/>
-      <c r="AO10" s="10"/>
+      <c r="AN10" s="15"/>
+      <c r="AO10" s="15"/>
+      <c r="AP10" s="15"/>
+      <c r="AQ10" s="16" t="str">
+        <f aca="false">IF(COUNT(AL10:AP10)=0,"",SUM(AL10:AP10))</f>
+        <v/>
+      </c>
+      <c r="AR10" s="17"/>
+      <c r="AS10" s="17"/>
+      <c r="AT10" s="17"/>
+      <c r="AU10" s="15"/>
+      <c r="AV10" s="15"/>
+      <c r="AW10" s="15"/>
+      <c r="AX10" s="15"/>
+      <c r="AY10" s="15"/>
+      <c r="AZ10" s="15"/>
+      <c r="BA10" s="15"/>
+      <c r="BB10" s="15"/>
+      <c r="BC10" s="15"/>
+      <c r="BD10" s="15"/>
+      <c r="BE10" s="15"/>
+      <c r="BF10" s="15"/>
+      <c r="BG10" s="15"/>
+      <c r="BH10" s="15"/>
+      <c r="BI10" s="15"/>
+      <c r="BJ10" s="15"/>
+      <c r="BK10" s="15"/>
+      <c r="BL10" s="15"/>
+      <c r="BM10" s="15"/>
+      <c r="BN10" s="15"/>
+      <c r="BO10" s="9"/>
+      <c r="BP10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9"/>
@@ -3962,14 +4666,44 @@
       <c r="AE11" s="12"/>
       <c r="AF11" s="10"/>
       <c r="AG11" s="12"/>
-      <c r="AH11" s="15"/>
-      <c r="AI11" s="15"/>
-      <c r="AJ11" s="15"/>
-      <c r="AK11" s="15"/>
+      <c r="AH11" s="10"/>
+      <c r="AI11" s="12"/>
+      <c r="AJ11" s="10"/>
+      <c r="AK11" s="12"/>
       <c r="AL11" s="15"/>
       <c r="AM11" s="15"/>
-      <c r="AN11" s="9"/>
-      <c r="AO11" s="10"/>
+      <c r="AN11" s="15"/>
+      <c r="AO11" s="15"/>
+      <c r="AP11" s="15"/>
+      <c r="AQ11" s="16" t="str">
+        <f aca="false">IF(COUNT(AL11:AP11)=0,"",SUM(AL11:AP11))</f>
+        <v/>
+      </c>
+      <c r="AR11" s="17"/>
+      <c r="AS11" s="17"/>
+      <c r="AT11" s="17"/>
+      <c r="AU11" s="15"/>
+      <c r="AV11" s="15"/>
+      <c r="AW11" s="15"/>
+      <c r="AX11" s="15"/>
+      <c r="AY11" s="15"/>
+      <c r="AZ11" s="15"/>
+      <c r="BA11" s="15"/>
+      <c r="BB11" s="15"/>
+      <c r="BC11" s="15"/>
+      <c r="BD11" s="15"/>
+      <c r="BE11" s="15"/>
+      <c r="BF11" s="15"/>
+      <c r="BG11" s="15"/>
+      <c r="BH11" s="15"/>
+      <c r="BI11" s="15"/>
+      <c r="BJ11" s="15"/>
+      <c r="BK11" s="15"/>
+      <c r="BL11" s="15"/>
+      <c r="BM11" s="15"/>
+      <c r="BN11" s="15"/>
+      <c r="BO11" s="9"/>
+      <c r="BP11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9"/>
@@ -4008,14 +4742,44 @@
       <c r="AE12" s="12"/>
       <c r="AF12" s="10"/>
       <c r="AG12" s="12"/>
-      <c r="AH12" s="15"/>
-      <c r="AI12" s="15"/>
-      <c r="AJ12" s="15"/>
-      <c r="AK12" s="15"/>
+      <c r="AH12" s="10"/>
+      <c r="AI12" s="12"/>
+      <c r="AJ12" s="10"/>
+      <c r="AK12" s="12"/>
       <c r="AL12" s="15"/>
       <c r="AM12" s="15"/>
-      <c r="AN12" s="9"/>
-      <c r="AO12" s="10"/>
+      <c r="AN12" s="15"/>
+      <c r="AO12" s="15"/>
+      <c r="AP12" s="15"/>
+      <c r="AQ12" s="16" t="str">
+        <f aca="false">IF(COUNT(AL12:AP12)=0,"",SUM(AL12:AP12))</f>
+        <v/>
+      </c>
+      <c r="AR12" s="17"/>
+      <c r="AS12" s="17"/>
+      <c r="AT12" s="17"/>
+      <c r="AU12" s="15"/>
+      <c r="AV12" s="15"/>
+      <c r="AW12" s="15"/>
+      <c r="AX12" s="15"/>
+      <c r="AY12" s="15"/>
+      <c r="AZ12" s="15"/>
+      <c r="BA12" s="15"/>
+      <c r="BB12" s="15"/>
+      <c r="BC12" s="15"/>
+      <c r="BD12" s="15"/>
+      <c r="BE12" s="15"/>
+      <c r="BF12" s="15"/>
+      <c r="BG12" s="15"/>
+      <c r="BH12" s="15"/>
+      <c r="BI12" s="15"/>
+      <c r="BJ12" s="15"/>
+      <c r="BK12" s="15"/>
+      <c r="BL12" s="15"/>
+      <c r="BM12" s="15"/>
+      <c r="BN12" s="15"/>
+      <c r="BO12" s="9"/>
+      <c r="BP12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9"/>
@@ -4054,14 +4818,44 @@
       <c r="AE13" s="12"/>
       <c r="AF13" s="10"/>
       <c r="AG13" s="12"/>
-      <c r="AH13" s="15"/>
-      <c r="AI13" s="15"/>
-      <c r="AJ13" s="15"/>
-      <c r="AK13" s="15"/>
+      <c r="AH13" s="10"/>
+      <c r="AI13" s="12"/>
+      <c r="AJ13" s="10"/>
+      <c r="AK13" s="12"/>
       <c r="AL13" s="15"/>
       <c r="AM13" s="15"/>
-      <c r="AN13" s="9"/>
-      <c r="AO13" s="10"/>
+      <c r="AN13" s="15"/>
+      <c r="AO13" s="15"/>
+      <c r="AP13" s="15"/>
+      <c r="AQ13" s="16" t="str">
+        <f aca="false">IF(COUNT(AL13:AP13)=0,"",SUM(AL13:AP13))</f>
+        <v/>
+      </c>
+      <c r="AR13" s="17"/>
+      <c r="AS13" s="17"/>
+      <c r="AT13" s="17"/>
+      <c r="AU13" s="15"/>
+      <c r="AV13" s="15"/>
+      <c r="AW13" s="15"/>
+      <c r="AX13" s="15"/>
+      <c r="AY13" s="15"/>
+      <c r="AZ13" s="15"/>
+      <c r="BA13" s="15"/>
+      <c r="BB13" s="15"/>
+      <c r="BC13" s="15"/>
+      <c r="BD13" s="15"/>
+      <c r="BE13" s="15"/>
+      <c r="BF13" s="15"/>
+      <c r="BG13" s="15"/>
+      <c r="BH13" s="15"/>
+      <c r="BI13" s="15"/>
+      <c r="BJ13" s="15"/>
+      <c r="BK13" s="15"/>
+      <c r="BL13" s="15"/>
+      <c r="BM13" s="15"/>
+      <c r="BN13" s="15"/>
+      <c r="BO13" s="9"/>
+      <c r="BP13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9"/>
@@ -4100,14 +4894,44 @@
       <c r="AE14" s="12"/>
       <c r="AF14" s="10"/>
       <c r="AG14" s="12"/>
-      <c r="AH14" s="15"/>
-      <c r="AI14" s="15"/>
-      <c r="AJ14" s="15"/>
-      <c r="AK14" s="15"/>
+      <c r="AH14" s="10"/>
+      <c r="AI14" s="12"/>
+      <c r="AJ14" s="10"/>
+      <c r="AK14" s="12"/>
       <c r="AL14" s="15"/>
       <c r="AM14" s="15"/>
-      <c r="AN14" s="9"/>
-      <c r="AO14" s="10"/>
+      <c r="AN14" s="15"/>
+      <c r="AO14" s="15"/>
+      <c r="AP14" s="15"/>
+      <c r="AQ14" s="16" t="str">
+        <f aca="false">IF(COUNT(AL14:AP14)=0,"",SUM(AL14:AP14))</f>
+        <v/>
+      </c>
+      <c r="AR14" s="17"/>
+      <c r="AS14" s="17"/>
+      <c r="AT14" s="17"/>
+      <c r="AU14" s="15"/>
+      <c r="AV14" s="15"/>
+      <c r="AW14" s="15"/>
+      <c r="AX14" s="15"/>
+      <c r="AY14" s="15"/>
+      <c r="AZ14" s="15"/>
+      <c r="BA14" s="15"/>
+      <c r="BB14" s="15"/>
+      <c r="BC14" s="15"/>
+      <c r="BD14" s="15"/>
+      <c r="BE14" s="15"/>
+      <c r="BF14" s="15"/>
+      <c r="BG14" s="15"/>
+      <c r="BH14" s="15"/>
+      <c r="BI14" s="15"/>
+      <c r="BJ14" s="15"/>
+      <c r="BK14" s="15"/>
+      <c r="BL14" s="15"/>
+      <c r="BM14" s="15"/>
+      <c r="BN14" s="15"/>
+      <c r="BO14" s="9"/>
+      <c r="BP14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9"/>
@@ -4146,14 +4970,44 @@
       <c r="AE15" s="12"/>
       <c r="AF15" s="10"/>
       <c r="AG15" s="12"/>
-      <c r="AH15" s="15"/>
-      <c r="AI15" s="15"/>
-      <c r="AJ15" s="15"/>
-      <c r="AK15" s="15"/>
+      <c r="AH15" s="10"/>
+      <c r="AI15" s="12"/>
+      <c r="AJ15" s="10"/>
+      <c r="AK15" s="12"/>
       <c r="AL15" s="15"/>
       <c r="AM15" s="15"/>
-      <c r="AN15" s="9"/>
-      <c r="AO15" s="10"/>
+      <c r="AN15" s="15"/>
+      <c r="AO15" s="15"/>
+      <c r="AP15" s="15"/>
+      <c r="AQ15" s="16" t="str">
+        <f aca="false">IF(COUNT(AL15:AP15)=0,"",SUM(AL15:AP15))</f>
+        <v/>
+      </c>
+      <c r="AR15" s="17"/>
+      <c r="AS15" s="17"/>
+      <c r="AT15" s="17"/>
+      <c r="AU15" s="15"/>
+      <c r="AV15" s="15"/>
+      <c r="AW15" s="15"/>
+      <c r="AX15" s="15"/>
+      <c r="AY15" s="15"/>
+      <c r="AZ15" s="15"/>
+      <c r="BA15" s="15"/>
+      <c r="BB15" s="15"/>
+      <c r="BC15" s="15"/>
+      <c r="BD15" s="15"/>
+      <c r="BE15" s="15"/>
+      <c r="BF15" s="15"/>
+      <c r="BG15" s="15"/>
+      <c r="BH15" s="15"/>
+      <c r="BI15" s="15"/>
+      <c r="BJ15" s="15"/>
+      <c r="BK15" s="15"/>
+      <c r="BL15" s="15"/>
+      <c r="BM15" s="15"/>
+      <c r="BN15" s="15"/>
+      <c r="BO15" s="9"/>
+      <c r="BP15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9"/>
@@ -4192,18 +5046,48 @@
       <c r="AE16" s="12"/>
       <c r="AF16" s="10"/>
       <c r="AG16" s="12"/>
-      <c r="AH16" s="15"/>
-      <c r="AI16" s="15"/>
-      <c r="AJ16" s="15"/>
-      <c r="AK16" s="15"/>
+      <c r="AH16" s="10"/>
+      <c r="AI16" s="12"/>
+      <c r="AJ16" s="10"/>
+      <c r="AK16" s="12"/>
       <c r="AL16" s="15"/>
       <c r="AM16" s="15"/>
-      <c r="AN16" s="9"/>
-      <c r="AO16" s="10"/>
+      <c r="AN16" s="15"/>
+      <c r="AO16" s="15"/>
+      <c r="AP16" s="15"/>
+      <c r="AQ16" s="16" t="str">
+        <f aca="false">IF(COUNT(AL16:AP16)=0,"",SUM(AL16:AP16))</f>
+        <v/>
+      </c>
+      <c r="AR16" s="17"/>
+      <c r="AS16" s="17"/>
+      <c r="AT16" s="17"/>
+      <c r="AU16" s="15"/>
+      <c r="AV16" s="15"/>
+      <c r="AW16" s="15"/>
+      <c r="AX16" s="15"/>
+      <c r="AY16" s="15"/>
+      <c r="AZ16" s="15"/>
+      <c r="BA16" s="15"/>
+      <c r="BB16" s="15"/>
+      <c r="BC16" s="15"/>
+      <c r="BD16" s="15"/>
+      <c r="BE16" s="15"/>
+      <c r="BF16" s="15"/>
+      <c r="BG16" s="15"/>
+      <c r="BH16" s="15"/>
+      <c r="BI16" s="15"/>
+      <c r="BJ16" s="15"/>
+      <c r="BK16" s="15"/>
+      <c r="BL16" s="15"/>
+      <c r="BM16" s="15"/>
+      <c r="BN16" s="15"/>
+      <c r="BO16" s="9"/>
+      <c r="BP16" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
-        <v>118</v>
+      <c r="A18" s="18" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -4260,7 +5144,7 @@
       <formula1>Lists!$E$2:$E$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="AO2:AO16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="BP2:BP16" type="list">
       <formula1>Lists!$E$2:$E$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4310,954 +5194,954 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="17" t="s">
+      <c r="A1" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>131</v>
+      <c r="C1" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="K1" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="I2" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="J2" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="K2" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>143</v>
+      <c r="A2" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="K2" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="M2" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="N2" s="20" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>154</v>
+      <c r="A3" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="M3" s="20" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="G4" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="J4" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="L4" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="M4" s="18" t="s">
-        <v>163</v>
+      <c r="A4" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="M4" s="20" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="M5" s="18" t="s">
-        <v>170</v>
+      <c r="A5" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="M5" s="20" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="M6" s="18" t="s">
-        <v>176</v>
+      <c r="A6" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="M6" s="20" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>177</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="M7" s="18" t="s">
-        <v>181</v>
+      <c r="A7" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="L7" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D8" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>184</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>185</v>
+      <c r="D8" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D9" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>189</v>
+      <c r="D9" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>191</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>192</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>193</v>
+      <c r="D10" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D11" s="18" t="s">
-        <v>194</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>197</v>
+      <c r="D11" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D12" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="G12" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="H12" s="18" t="s">
-        <v>200</v>
+      <c r="D12" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F13" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G13" s="18" t="s">
-        <v>202</v>
-      </c>
-      <c r="H13" s="18" t="s">
-        <v>203</v>
+      <c r="F13" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="G14" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="H14" s="18" t="s">
-        <v>206</v>
+      <c r="F14" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F15" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="G15" s="18" t="s">
-        <v>208</v>
-      </c>
-      <c r="H15" s="18" t="s">
-        <v>209</v>
+      <c r="F15" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F16" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="H16" s="18" t="s">
-        <v>212</v>
+      <c r="F16" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F17" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="G17" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="H17" s="18" t="s">
-        <v>215</v>
+      <c r="F17" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F18" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="G18" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="H18" s="18" t="s">
-        <v>218</v>
+      <c r="F18" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F19" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="G19" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="H19" s="18" t="s">
-        <v>221</v>
+      <c r="F19" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F20" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="G20" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>224</v>
+      <c r="F20" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F21" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="H21" s="18" t="s">
-        <v>227</v>
+      <c r="F21" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="H21" s="20" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F22" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="H22" s="18" t="s">
-        <v>230</v>
+      <c r="F22" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="H22" s="20" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G23" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="H23" s="18" t="s">
-        <v>232</v>
+      <c r="G23" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G24" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="H24" s="18" t="s">
-        <v>234</v>
+      <c r="G24" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G25" s="18" t="s">
-        <v>235</v>
-      </c>
-      <c r="H25" s="18" t="s">
-        <v>236</v>
+      <c r="G25" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G26" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="H26" s="18" t="s">
-        <v>238</v>
+      <c r="G26" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="H26" s="20" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G27" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="H27" s="18" t="s">
-        <v>240</v>
+      <c r="G27" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="H27" s="20" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="H28" s="18" t="s">
-        <v>242</v>
+      <c r="G28" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="H28" s="20" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G29" s="18" t="s">
-        <v>243</v>
-      </c>
-      <c r="H29" s="18" t="s">
-        <v>244</v>
+      <c r="G29" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="H29" s="20" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G30" s="18" t="s">
-        <v>245</v>
-      </c>
-      <c r="H30" s="18" t="s">
-        <v>246</v>
+      <c r="G30" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G31" s="18" t="s">
-        <v>247</v>
-      </c>
-      <c r="H31" s="18" t="s">
-        <v>248</v>
+      <c r="G31" s="20" t="s">
+        <v>286</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G32" s="18" t="s">
-        <v>249</v>
-      </c>
-      <c r="H32" s="18" t="s">
-        <v>250</v>
+      <c r="G32" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="18" t="s">
-        <v>251</v>
-      </c>
-      <c r="H33" s="18" t="s">
-        <v>252</v>
+      <c r="G33" s="20" t="s">
+        <v>290</v>
+      </c>
+      <c r="H33" s="20" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G34" s="18" t="s">
-        <v>253</v>
-      </c>
-      <c r="H34" s="18" t="s">
-        <v>254</v>
+      <c r="G34" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G35" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="H35" s="18" t="s">
-        <v>256</v>
+      <c r="G35" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="H35" s="20" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G36" s="18" t="s">
-        <v>257</v>
-      </c>
-      <c r="H36" s="18" t="s">
-        <v>258</v>
+      <c r="G36" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="H36" s="20" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G37" s="18" t="s">
-        <v>259</v>
-      </c>
-      <c r="H37" s="18" t="s">
-        <v>260</v>
+      <c r="G37" s="20" t="s">
+        <v>298</v>
+      </c>
+      <c r="H37" s="20" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G38" s="18" t="s">
-        <v>261</v>
-      </c>
-      <c r="H38" s="18" t="s">
-        <v>262</v>
+      <c r="G38" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="H38" s="20" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G39" s="18" t="s">
-        <v>263</v>
-      </c>
-      <c r="H39" s="18" t="s">
-        <v>264</v>
+      <c r="G39" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="H39" s="20" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G40" s="18" t="s">
-        <v>265</v>
-      </c>
-      <c r="H40" s="18" t="s">
-        <v>266</v>
+      <c r="G40" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="H40" s="20" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G41" s="18" t="s">
-        <v>267</v>
-      </c>
-      <c r="H41" s="18" t="s">
-        <v>268</v>
+      <c r="G41" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="H41" s="20" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G42" s="18" t="s">
-        <v>269</v>
-      </c>
-      <c r="H42" s="18" t="s">
-        <v>270</v>
+      <c r="G42" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="H42" s="20" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G43" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="H43" s="18" t="s">
-        <v>272</v>
+      <c r="G43" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="H43" s="20" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G44" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="H44" s="18" t="s">
-        <v>274</v>
+      <c r="G44" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="H44" s="20" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G45" s="18" t="s">
-        <v>275</v>
-      </c>
-      <c r="H45" s="18" t="s">
-        <v>276</v>
+      <c r="G45" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="H45" s="20" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G46" s="18" t="s">
-        <v>277</v>
-      </c>
-      <c r="H46" s="18" t="s">
-        <v>278</v>
+      <c r="G46" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="H46" s="20" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G47" s="18" t="s">
-        <v>279</v>
-      </c>
-      <c r="H47" s="18" t="s">
-        <v>280</v>
+      <c r="G47" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="H47" s="20" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G48" s="18" t="s">
-        <v>281</v>
-      </c>
-      <c r="H48" s="18" t="s">
-        <v>282</v>
+      <c r="G48" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="H48" s="20" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G49" s="18" t="s">
-        <v>283</v>
-      </c>
-      <c r="H49" s="18" t="s">
-        <v>284</v>
+      <c r="G49" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="H49" s="20" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G50" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="H50" s="18" t="s">
-        <v>286</v>
+      <c r="G50" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="H50" s="20" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G51" s="18" t="s">
-        <v>287</v>
-      </c>
-      <c r="H51" s="18" t="s">
-        <v>288</v>
+      <c r="G51" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="H51" s="20" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G52" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="H52" s="18" t="s">
-        <v>290</v>
+      <c r="G52" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="H52" s="20" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G53" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="H53" s="18" t="s">
-        <v>292</v>
+      <c r="G53" s="20" t="s">
+        <v>330</v>
+      </c>
+      <c r="H53" s="20" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G54" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="H54" s="18" t="s">
-        <v>294</v>
+      <c r="G54" s="20" t="s">
+        <v>332</v>
+      </c>
+      <c r="H54" s="20" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G55" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="H55" s="18" t="s">
-        <v>296</v>
+      <c r="G55" s="20" t="s">
+        <v>334</v>
+      </c>
+      <c r="H55" s="20" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G56" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="H56" s="18" t="s">
-        <v>298</v>
+      <c r="G56" s="20" t="s">
+        <v>336</v>
+      </c>
+      <c r="H56" s="20" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G57" s="18" t="s">
-        <v>299</v>
-      </c>
-      <c r="H57" s="18" t="s">
-        <v>300</v>
+      <c r="G57" s="20" t="s">
+        <v>338</v>
+      </c>
+      <c r="H57" s="20" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G58" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="H58" s="18" t="s">
-        <v>302</v>
+      <c r="G58" s="20" t="s">
+        <v>340</v>
+      </c>
+      <c r="H58" s="20" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G59" s="18" t="s">
-        <v>303</v>
-      </c>
-      <c r="H59" s="18" t="s">
-        <v>304</v>
+      <c r="G59" s="20" t="s">
+        <v>342</v>
+      </c>
+      <c r="H59" s="20" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G60" s="18" t="s">
-        <v>305</v>
-      </c>
-      <c r="H60" s="18" t="s">
-        <v>306</v>
+      <c r="G60" s="20" t="s">
+        <v>344</v>
+      </c>
+      <c r="H60" s="20" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G61" s="18" t="s">
-        <v>307</v>
-      </c>
-      <c r="H61" s="18" t="s">
-        <v>308</v>
+      <c r="G61" s="20" t="s">
+        <v>346</v>
+      </c>
+      <c r="H61" s="20" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G62" s="18" t="s">
-        <v>309</v>
-      </c>
-      <c r="H62" s="18" t="s">
-        <v>310</v>
+      <c r="G62" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="H62" s="20" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G63" s="18" t="s">
-        <v>311</v>
-      </c>
-      <c r="H63" s="18" t="s">
-        <v>312</v>
+      <c r="G63" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="H63" s="20" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G64" s="18" t="s">
-        <v>313</v>
-      </c>
-      <c r="H64" s="18" t="s">
-        <v>314</v>
+      <c r="G64" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="H64" s="20" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G65" s="18" t="s">
-        <v>315</v>
-      </c>
-      <c r="H65" s="18" t="s">
-        <v>316</v>
+      <c r="G65" s="20" t="s">
+        <v>354</v>
+      </c>
+      <c r="H65" s="20" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G66" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="H66" s="18" t="s">
-        <v>318</v>
+      <c r="G66" s="20" t="s">
+        <v>356</v>
+      </c>
+      <c r="H66" s="20" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G67" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="H67" s="18" t="s">
-        <v>320</v>
+      <c r="G67" s="20" t="s">
+        <v>358</v>
+      </c>
+      <c r="H67" s="20" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G68" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="H68" s="18" t="s">
-        <v>322</v>
+      <c r="G68" s="20" t="s">
+        <v>360</v>
+      </c>
+      <c r="H68" s="20" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G69" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="H69" s="18" t="s">
-        <v>324</v>
+      <c r="G69" s="20" t="s">
+        <v>362</v>
+      </c>
+      <c r="H69" s="20" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G70" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="H70" s="18" t="s">
-        <v>326</v>
+      <c r="G70" s="20" t="s">
+        <v>364</v>
+      </c>
+      <c r="H70" s="20" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G71" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="H71" s="18" t="s">
-        <v>328</v>
+      <c r="G71" s="20" t="s">
+        <v>366</v>
+      </c>
+      <c r="H71" s="20" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G72" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="H72" s="18" t="s">
-        <v>330</v>
+      <c r="G72" s="20" t="s">
+        <v>368</v>
+      </c>
+      <c r="H72" s="20" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G73" s="18" t="s">
-        <v>331</v>
-      </c>
-      <c r="H73" s="18" t="s">
-        <v>332</v>
+      <c r="G73" s="20" t="s">
+        <v>370</v>
+      </c>
+      <c r="H73" s="20" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G74" s="18" t="s">
-        <v>333</v>
-      </c>
-      <c r="H74" s="18" t="s">
-        <v>334</v>
+      <c r="G74" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="H74" s="20" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G75" s="18" t="s">
-        <v>335</v>
-      </c>
-      <c r="H75" s="18" t="s">
-        <v>336</v>
+      <c r="G75" s="20" t="s">
+        <v>374</v>
+      </c>
+      <c r="H75" s="20" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G76" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="H76" s="18" t="s">
-        <v>338</v>
+      <c r="G76" s="20" t="s">
+        <v>376</v>
+      </c>
+      <c r="H76" s="20" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G77" s="18" t="s">
-        <v>339</v>
-      </c>
-      <c r="H77" s="18" t="s">
-        <v>340</v>
+      <c r="G77" s="20" t="s">
+        <v>378</v>
+      </c>
+      <c r="H77" s="20" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G78" s="18" t="s">
-        <v>341</v>
-      </c>
-      <c r="H78" s="18" t="s">
-        <v>342</v>
+      <c r="G78" s="20" t="s">
+        <v>380</v>
+      </c>
+      <c r="H78" s="20" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G79" s="18" t="s">
-        <v>343</v>
-      </c>
-      <c r="H79" s="18" t="s">
-        <v>344</v>
+      <c r="G79" s="20" t="s">
+        <v>382</v>
+      </c>
+      <c r="H79" s="20" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H80" s="18" t="s">
-        <v>345</v>
+      <c r="H80" s="20" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H81" s="18" t="s">
-        <v>346</v>
+      <c r="H81" s="20" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H82" s="18" t="s">
-        <v>347</v>
+      <c r="H82" s="20" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H83" s="18" t="s">
-        <v>348</v>
+      <c r="H83" s="20" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H84" s="18" t="s">
-        <v>349</v>
+      <c r="H84" s="20" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H85" s="18" t="s">
-        <v>350</v>
+      <c r="H85" s="20" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H86" s="18" t="s">
-        <v>351</v>
+      <c r="H86" s="20" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H87" s="18" t="s">
-        <v>352</v>
+      <c r="H87" s="20" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H88" s="18" t="s">
-        <v>353</v>
+      <c r="H88" s="20" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H89" s="18" t="s">
-        <v>354</v>
+      <c r="H89" s="20" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H90" s="18" t="s">
-        <v>355</v>
+      <c r="H90" s="20" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H91" s="18" t="s">
-        <v>356</v>
+      <c r="H91" s="20" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H92" s="18" t="s">
-        <v>357</v>
+      <c r="H92" s="20" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H93" s="18" t="s">
-        <v>358</v>
+      <c r="H93" s="20" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H94" s="18" t="s">
-        <v>359</v>
+      <c r="H94" s="20" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H95" s="18" t="s">
-        <v>360</v>
+      <c r="H95" s="20" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H96" s="18" t="s">
-        <v>361</v>
+      <c r="H96" s="20" t="s">
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -5284,665 +6168,665 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>362</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>363</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>364</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>365</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>366</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>367</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>368</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>369</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>370</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>371</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>372</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>373</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>374</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>375</v>
-      </c>
-      <c r="O1" s="17" t="s">
-        <v>376</v>
-      </c>
-      <c r="P1" s="17" t="s">
-        <v>377</v>
-      </c>
-      <c r="Q1" s="17" t="s">
-        <v>378</v>
-      </c>
-      <c r="R1" s="17" t="s">
-        <v>379</v>
+      <c r="A1" s="19" t="s">
+        <v>401</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>402</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>403</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>404</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>405</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>406</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>407</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>409</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="K1" s="19" t="s">
+        <v>411</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>412</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>413</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>414</v>
+      </c>
+      <c r="O1" s="19" t="s">
+        <v>415</v>
+      </c>
+      <c r="P1" s="19" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>417</v>
+      </c>
+      <c r="R1" s="19" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
-        <v>380</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>382</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>384</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>385</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>386</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>387</v>
-      </c>
-      <c r="I2" s="18" t="s">
-        <v>388</v>
-      </c>
-      <c r="J2" s="18" t="s">
-        <v>389</v>
-      </c>
-      <c r="K2" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>391</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>392</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>394</v>
-      </c>
-      <c r="P2" s="18" t="s">
-        <v>395</v>
-      </c>
-      <c r="Q2" s="18" t="s">
-        <v>396</v>
-      </c>
-      <c r="R2" s="18" t="s">
-        <v>397</v>
+      <c r="A2" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>422</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>423</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>424</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>426</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>427</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>428</v>
+      </c>
+      <c r="K2" s="20" t="s">
+        <v>429</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>430</v>
+      </c>
+      <c r="M2" s="20" t="s">
+        <v>431</v>
+      </c>
+      <c r="N2" s="20" t="s">
+        <v>432</v>
+      </c>
+      <c r="O2" s="20" t="s">
+        <v>433</v>
+      </c>
+      <c r="P2" s="20" t="s">
+        <v>434</v>
+      </c>
+      <c r="Q2" s="20" t="s">
+        <v>435</v>
+      </c>
+      <c r="R2" s="20" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>398</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>399</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>400</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>401</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>402</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>403</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>404</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>405</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>406</v>
-      </c>
-      <c r="J3" s="18" t="s">
+      <c r="A3" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>438</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>439</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>440</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>441</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>442</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>443</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>444</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>446</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="M3" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="N3" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="O3" s="20" t="s">
+        <v>451</v>
+      </c>
+      <c r="P3" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="Q3" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="R3" s="20" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="20" t="s">
+        <v>455</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>456</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>458</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>459</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>460</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>462</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>463</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>464</v>
+      </c>
+      <c r="K4" s="20" t="s">
+        <v>465</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>466</v>
+      </c>
+      <c r="M4" s="20" t="s">
+        <v>467</v>
+      </c>
+      <c r="N4" s="20" t="s">
+        <v>468</v>
+      </c>
+      <c r="O4" s="20" t="s">
+        <v>469</v>
+      </c>
+      <c r="P4" s="20" t="s">
+        <v>470</v>
+      </c>
+      <c r="Q4" s="20" t="s">
+        <v>471</v>
+      </c>
+      <c r="R4" s="20" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
+        <v>473</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>474</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>475</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>476</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>477</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>478</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>407</v>
       </c>
-      <c r="K3" s="18" t="s">
-        <v>408</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="N3" s="18" t="s">
-        <v>411</v>
-      </c>
-      <c r="O3" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="P3" s="18" t="s">
+      <c r="H5" s="20" t="s">
+        <v>479</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>480</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>481</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>482</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>483</v>
+      </c>
+      <c r="M5" s="20" t="s">
+        <v>484</v>
+      </c>
+      <c r="N5" s="20" t="s">
+        <v>485</v>
+      </c>
+      <c r="O5" s="20" t="s">
+        <v>486</v>
+      </c>
+      <c r="P5" s="20" t="s">
+        <v>487</v>
+      </c>
+      <c r="Q5" s="20" t="s">
+        <v>488</v>
+      </c>
+      <c r="R5" s="20" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
+        <v>490</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>491</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>492</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>493</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>494</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>495</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>496</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>497</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>498</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>499</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>500</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>501</v>
+      </c>
+      <c r="M6" s="20" t="s">
         <v>413</v>
       </c>
-      <c r="Q3" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="R3" s="18" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>416</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>417</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>418</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>419</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>420</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>421</v>
-      </c>
-      <c r="G4" s="18" t="s">
-        <v>422</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>423</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>424</v>
-      </c>
-      <c r="J4" s="18" t="s">
-        <v>425</v>
-      </c>
-      <c r="K4" s="18" t="s">
-        <v>426</v>
-      </c>
-      <c r="L4" s="18" t="s">
+      <c r="N6" s="20" t="s">
+        <v>502</v>
+      </c>
+      <c r="O6" s="20" t="s">
+        <v>503</v>
+      </c>
+      <c r="P6" s="20" t="s">
+        <v>504</v>
+      </c>
+      <c r="Q6" s="20" t="s">
+        <v>505</v>
+      </c>
+      <c r="R6" s="20" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>507</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>509</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>510</v>
+      </c>
+      <c r="E7" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="M4" s="18" t="s">
-        <v>428</v>
-      </c>
-      <c r="N4" s="18" t="s">
-        <v>429</v>
-      </c>
-      <c r="O4" s="18" t="s">
-        <v>430</v>
-      </c>
-      <c r="P4" s="18" t="s">
-        <v>431</v>
-      </c>
-      <c r="Q4" s="18" t="s">
-        <v>432</v>
-      </c>
-      <c r="R4" s="18" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>434</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>435</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>436</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>437</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>438</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>439</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>368</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>440</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>441</v>
-      </c>
-      <c r="J5" s="18" t="s">
-        <v>442</v>
-      </c>
-      <c r="K5" s="18" t="s">
-        <v>443</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>444</v>
-      </c>
-      <c r="M5" s="18" t="s">
-        <v>445</v>
-      </c>
-      <c r="N5" s="18" t="s">
-        <v>446</v>
-      </c>
-      <c r="O5" s="18" t="s">
-        <v>447</v>
-      </c>
-      <c r="P5" s="18" t="s">
-        <v>448</v>
-      </c>
-      <c r="Q5" s="18" t="s">
-        <v>449</v>
-      </c>
-      <c r="R5" s="18" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>451</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>452</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>453</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>454</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>455</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>456</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>457</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>458</v>
-      </c>
-      <c r="I6" s="18" t="s">
-        <v>459</v>
-      </c>
-      <c r="J6" s="18" t="s">
-        <v>460</v>
-      </c>
-      <c r="K6" s="18" t="s">
-        <v>461</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>462</v>
-      </c>
-      <c r="M6" s="18" t="s">
-        <v>374</v>
-      </c>
-      <c r="N6" s="18" t="s">
-        <v>463</v>
-      </c>
-      <c r="O6" s="18" t="s">
-        <v>464</v>
-      </c>
-      <c r="P6" s="18" t="s">
-        <v>465</v>
-      </c>
-      <c r="Q6" s="18" t="s">
-        <v>466</v>
-      </c>
-      <c r="R6" s="18" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>468</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>469</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>470</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>471</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>388</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>472</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>473</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>474</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>475</v>
-      </c>
-      <c r="J7" s="18" t="s">
-        <v>476</v>
-      </c>
-      <c r="K7" s="18" t="s">
-        <v>477</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>478</v>
-      </c>
-      <c r="M7" s="18" t="s">
-        <v>479</v>
-      </c>
-      <c r="N7" s="18" t="s">
-        <v>480</v>
-      </c>
-      <c r="O7" s="18" t="s">
-        <v>481</v>
-      </c>
-      <c r="P7" s="18" t="s">
-        <v>482</v>
-      </c>
-      <c r="Q7" s="18" t="s">
-        <v>483</v>
-      </c>
-      <c r="R7" s="18" t="s">
-        <v>484</v>
+      <c r="F7" s="20" t="s">
+        <v>511</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>512</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>513</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>514</v>
+      </c>
+      <c r="J7" s="20" t="s">
+        <v>515</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>516</v>
+      </c>
+      <c r="L7" s="20" t="s">
+        <v>517</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>518</v>
+      </c>
+      <c r="N7" s="20" t="s">
+        <v>519</v>
+      </c>
+      <c r="O7" s="20" t="s">
+        <v>520</v>
+      </c>
+      <c r="P7" s="20" t="s">
+        <v>521</v>
+      </c>
+      <c r="Q7" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="R7" s="20" t="s">
+        <v>523</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>485</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>486</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>487</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>488</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>489</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>490</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>491</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>492</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>493</v>
-      </c>
-      <c r="J8" s="18" t="s">
-        <v>494</v>
-      </c>
-      <c r="K8" s="18" t="s">
-        <v>495</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>496</v>
-      </c>
-      <c r="M8" s="18" t="s">
-        <v>497</v>
-      </c>
-      <c r="N8" s="18" t="s">
-        <v>498</v>
-      </c>
-      <c r="O8" s="18" t="s">
-        <v>499</v>
-      </c>
-      <c r="P8" s="18" t="s">
-        <v>500</v>
-      </c>
-      <c r="Q8" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="R8" s="18" t="s">
-        <v>502</v>
+      <c r="A8" s="20" t="s">
+        <v>524</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>525</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>526</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>527</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>528</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>529</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>530</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>531</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>532</v>
+      </c>
+      <c r="J8" s="20" t="s">
+        <v>533</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>534</v>
+      </c>
+      <c r="L8" s="20" t="s">
+        <v>535</v>
+      </c>
+      <c r="M8" s="20" t="s">
+        <v>536</v>
+      </c>
+      <c r="N8" s="20" t="s">
+        <v>537</v>
+      </c>
+      <c r="O8" s="20" t="s">
+        <v>538</v>
+      </c>
+      <c r="P8" s="20" t="s">
+        <v>539</v>
+      </c>
+      <c r="Q8" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="R8" s="20" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>503</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>504</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>505</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>507</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>508</v>
-      </c>
-      <c r="I9" s="18" t="s">
-        <v>509</v>
-      </c>
-      <c r="K9" s="18" t="s">
-        <v>510</v>
-      </c>
-      <c r="N9" s="18" t="s">
-        <v>511</v>
-      </c>
-      <c r="O9" s="18" t="s">
-        <v>512</v>
-      </c>
-      <c r="P9" s="18" t="s">
-        <v>513</v>
-      </c>
-      <c r="Q9" s="18" t="s">
-        <v>514</v>
-      </c>
-      <c r="R9" s="18" t="s">
-        <v>515</v>
+      <c r="A9" s="20" t="s">
+        <v>542</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>543</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>544</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>545</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>546</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>547</v>
+      </c>
+      <c r="I9" s="20" t="s">
+        <v>548</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="N9" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="O9" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="P9" s="20" t="s">
+        <v>552</v>
+      </c>
+      <c r="Q9" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="R9" s="20" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="18" t="s">
-        <v>516</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>517</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>518</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>519</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>520</v>
-      </c>
-      <c r="K10" s="18" t="s">
-        <v>521</v>
-      </c>
-      <c r="N10" s="18" t="s">
-        <v>522</v>
-      </c>
-      <c r="O10" s="18" t="s">
-        <v>523</v>
-      </c>
-      <c r="Q10" s="18" t="s">
-        <v>524</v>
-      </c>
-      <c r="R10" s="18" t="s">
-        <v>525</v>
+      <c r="C10" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>556</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>557</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>558</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>559</v>
+      </c>
+      <c r="K10" s="20" t="s">
+        <v>560</v>
+      </c>
+      <c r="N10" s="20" t="s">
+        <v>561</v>
+      </c>
+      <c r="O10" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="Q10" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="R10" s="20" t="s">
+        <v>564</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E11" s="18" t="s">
-        <v>526</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>527</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>528</v>
-      </c>
-      <c r="K11" s="18" t="s">
-        <v>529</v>
-      </c>
-      <c r="N11" s="18" t="s">
-        <v>530</v>
-      </c>
-      <c r="O11" s="18" t="s">
-        <v>531</v>
-      </c>
-      <c r="Q11" s="18" t="s">
-        <v>532</v>
+      <c r="E11" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>567</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="N11" s="20" t="s">
+        <v>569</v>
+      </c>
+      <c r="O11" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="Q11" s="20" t="s">
+        <v>571</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E12" s="18" t="s">
-        <v>533</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>534</v>
-      </c>
-      <c r="H12" s="18" t="s">
-        <v>535</v>
-      </c>
-      <c r="N12" s="18" t="s">
-        <v>536</v>
-      </c>
-      <c r="O12" s="18" t="s">
-        <v>537</v>
-      </c>
-      <c r="Q12" s="18" t="s">
-        <v>538</v>
+      <c r="E12" s="20" t="s">
+        <v>572</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>573</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="N12" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="O12" s="20" t="s">
+        <v>576</v>
+      </c>
+      <c r="Q12" s="20" t="s">
+        <v>577</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F13" s="18" t="s">
-        <v>539</v>
-      </c>
-      <c r="H13" s="18" t="s">
-        <v>540</v>
-      </c>
-      <c r="N13" s="18" t="s">
-        <v>541</v>
-      </c>
-      <c r="O13" s="18" t="s">
-        <v>542</v>
-      </c>
-      <c r="Q13" s="18" t="s">
-        <v>543</v>
+      <c r="F13" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="N13" s="20" t="s">
+        <v>580</v>
+      </c>
+      <c r="O13" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q13" s="20" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H14" s="18" t="s">
-        <v>544</v>
-      </c>
-      <c r="N14" s="18" t="s">
-        <v>545</v>
-      </c>
-      <c r="O14" s="18" t="s">
-        <v>546</v>
-      </c>
-      <c r="Q14" s="18" t="s">
-        <v>547</v>
+      <c r="H14" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="Q14" s="20" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H15" s="18" t="s">
-        <v>548</v>
-      </c>
-      <c r="N15" s="18" t="s">
-        <v>549</v>
-      </c>
-      <c r="O15" s="18" t="s">
-        <v>550</v>
-      </c>
-      <c r="Q15" s="18" t="s">
-        <v>551</v>
+      <c r="H15" s="20" t="s">
+        <v>587</v>
+      </c>
+      <c r="N15" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="O15" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="Q15" s="20" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H16" s="18" t="s">
-        <v>552</v>
-      </c>
-      <c r="N16" s="18" t="s">
-        <v>553</v>
-      </c>
-      <c r="O16" s="18" t="s">
-        <v>554</v>
+      <c r="H16" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H17" s="18" t="s">
-        <v>555</v>
-      </c>
-      <c r="N17" s="18" t="s">
-        <v>556</v>
-      </c>
-      <c r="O17" s="18" t="s">
-        <v>557</v>
+      <c r="H17" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="N17" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="O17" s="20" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H18" s="18" t="s">
-        <v>558</v>
-      </c>
-      <c r="N18" s="18" t="s">
-        <v>559</v>
-      </c>
-      <c r="O18" s="18" t="s">
-        <v>560</v>
+      <c r="H18" s="20" t="s">
+        <v>597</v>
+      </c>
+      <c r="N18" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="O18" s="20" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N19" s="18" t="s">
-        <v>561</v>
+      <c r="N19" s="20" t="s">
+        <v>600</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N20" s="18" t="s">
-        <v>562</v>
+      <c r="N20" s="20" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N21" s="18" t="s">
-        <v>563</v>
+      <c r="N21" s="20" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N22" s="18" t="s">
-        <v>564</v>
+      <c r="N22" s="20" t="s">
+        <v>603</v>
       </c>
     </row>
   </sheetData>

</xml_diff>